<commit_message>
new datasets and updated code
</commit_message>
<xml_diff>
--- a/data/2024_Falcinellli_Collabra.xlsx
+++ b/data/2024_Falcinellli_Collabra.xlsx
@@ -1,27 +1,27 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="10211"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="10419"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ileniafalcinelli/Desktop/revisions_TECo_scripts/Revisioni Preprint prima del RID per ESM/analisi_nuove/Cronbach's alphas, database, demo info/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/erinbuchanan/GitHub/Research/2_projects/Maria-Familiarity/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{202CD2F0-FB1B-DE4E-A14C-F528BB7996D3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8E602EFB-A454-1A4C-B240-3FB51899560B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4680" yWindow="500" windowWidth="28800" windowHeight="16400" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1440" yWindow="660" windowWidth="28800" windowHeight="16400" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="legenda" sheetId="2" r:id="rId1"/>
-    <sheet name="database" sheetId="1" r:id="rId2"/>
+    <sheet name="database" sheetId="1" r:id="rId1"/>
+    <sheet name="legenda" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="124519"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="879" uniqueCount="546">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="879" uniqueCount="636">
   <si>
     <t>Target_Word_ITA</t>
   </si>
@@ -1659,6 +1659,276 @@
   </si>
   <si>
     <t>The mean of Frequency ratings. It refers to the subjective perception of frequency of use of each Target Word.</t>
+  </si>
+  <si>
+    <t>word_italian</t>
+  </si>
+  <si>
+    <t>translation_word_english</t>
+  </si>
+  <si>
+    <t>category</t>
+  </si>
+  <si>
+    <t>concrete_mean</t>
+  </si>
+  <si>
+    <t>concrete_sd</t>
+  </si>
+  <si>
+    <t>action_effector_mean</t>
+  </si>
+  <si>
+    <t>action_effector_sd</t>
+  </si>
+  <si>
+    <t>action_effector_feet_mean</t>
+  </si>
+  <si>
+    <t>action_effector_feet_sd</t>
+  </si>
+  <si>
+    <t>action_effector_hands_mean</t>
+  </si>
+  <si>
+    <t>action_effector_hands_sd</t>
+  </si>
+  <si>
+    <t>action_effector_mouth_mean</t>
+  </si>
+  <si>
+    <t>action_effector_mouth_sd</t>
+  </si>
+  <si>
+    <t>action_effector_torso_mean</t>
+  </si>
+  <si>
+    <t>action_effector_torso_sd</t>
+  </si>
+  <si>
+    <t>arousal_mean</t>
+  </si>
+  <si>
+    <t>arousal_sd</t>
+  </si>
+  <si>
+    <t>aoa_mean</t>
+  </si>
+  <si>
+    <t>aoa_sd</t>
+  </si>
+  <si>
+    <t>body_object_interact_mean</t>
+  </si>
+  <si>
+    <t>body_object_interact_sd</t>
+  </si>
+  <si>
+    <t>context_avail_mean</t>
+  </si>
+  <si>
+    <t>context_avail_sd</t>
+  </si>
+  <si>
+    <t>expert_confidence_mean</t>
+  </si>
+  <si>
+    <t>expert_confidence_sd</t>
+  </si>
+  <si>
+    <t>dominance_mean</t>
+  </si>
+  <si>
+    <t>dominance_sd</t>
+  </si>
+  <si>
+    <t>emotional_mean</t>
+  </si>
+  <si>
+    <t>emotional_sd</t>
+  </si>
+  <si>
+    <t>convo_ease_mean</t>
+  </si>
+  <si>
+    <t>convo_ease_sd</t>
+  </si>
+  <si>
+    <t>expert_social_meta_mean</t>
+  </si>
+  <si>
+    <t>expert_social_meta_sd</t>
+  </si>
+  <si>
+    <t>define_ease_mean</t>
+  </si>
+  <si>
+    <t>define_ease_sd</t>
+  </si>
+  <si>
+    <t>familiar_mean</t>
+  </si>
+  <si>
+    <t>familiar_sd</t>
+  </si>
+  <si>
+    <t>freq_subjective_mean</t>
+  </si>
+  <si>
+    <t>freq_subjective_sd</t>
+  </si>
+  <si>
+    <t>freq_objective</t>
+  </si>
+  <si>
+    <t>imagine_mean</t>
+  </si>
+  <si>
+    <t>imagine_sd</t>
+  </si>
+  <si>
+    <t>interoception_mean</t>
+  </si>
+  <si>
+    <t>interoception_sd</t>
+  </si>
+  <si>
+    <t>metacognition_mean</t>
+  </si>
+  <si>
+    <t>metacognition_sd</t>
+  </si>
+  <si>
+    <t>modality_acquis_mean</t>
+  </si>
+  <si>
+    <t>modality_acquis_sd</t>
+  </si>
+  <si>
+    <t>natural_artific_mean</t>
+  </si>
+  <si>
+    <t>natural_artific_sd</t>
+  </si>
+  <si>
+    <t>open_negotiation_mean</t>
+  </si>
+  <si>
+    <t>open_negotiation_sd</t>
+  </si>
+  <si>
+    <t>perceived_distance_mean</t>
+  </si>
+  <si>
+    <t>perceived_distance_sd</t>
+  </si>
+  <si>
+    <t>personal_experience_mean</t>
+  </si>
+  <si>
+    <t>personal_experience_sd</t>
+  </si>
+  <si>
+    <t>perceived_impact_mean</t>
+  </si>
+  <si>
+    <t>perceived_impact_sd</t>
+  </si>
+  <si>
+    <t>perceived_impact_future_mean</t>
+  </si>
+  <si>
+    <t>perceived_impact_future_sd</t>
+  </si>
+  <si>
+    <t>perceived_impact_past_mean</t>
+  </si>
+  <si>
+    <t>perceived_impact_past_sd</t>
+  </si>
+  <si>
+    <t>perceived_impact_present_mean</t>
+  </si>
+  <si>
+    <t>perceived_impact_present_sd</t>
+  </si>
+  <si>
+    <t>political_relev_mean</t>
+  </si>
+  <si>
+    <t>political_relev_sd</t>
+  </si>
+  <si>
+    <t>percept_strength_mean</t>
+  </si>
+  <si>
+    <t>percept_strength_sd</t>
+  </si>
+  <si>
+    <t>percept_strength_hearing_mean</t>
+  </si>
+  <si>
+    <t>percept_strength_hearing_sd</t>
+  </si>
+  <si>
+    <t>percept_strength_smell_mean</t>
+  </si>
+  <si>
+    <t>percept_strength_smell_sd</t>
+  </si>
+  <si>
+    <t>percept_strength_taste_mean</t>
+  </si>
+  <si>
+    <t>percept_strength_taste_sd</t>
+  </si>
+  <si>
+    <t>percept_strength_touch_mean</t>
+  </si>
+  <si>
+    <t>percept_strength_touch_sd</t>
+  </si>
+  <si>
+    <t>percept_strength_vision_mean</t>
+  </si>
+  <si>
+    <t>percept_strength_vision_sd</t>
+  </si>
+  <si>
+    <t>scientificity_mean</t>
+  </si>
+  <si>
+    <t>scientificity_sd</t>
+  </si>
+  <si>
+    <t>social_meta_mean</t>
+  </si>
+  <si>
+    <t>social_meta_sd</t>
+  </si>
+  <si>
+    <t>social_valence_mean</t>
+  </si>
+  <si>
+    <t>social_valence_sd</t>
+  </si>
+  <si>
+    <t>valence_mean</t>
+  </si>
+  <si>
+    <t>valence_sd</t>
+  </si>
+  <si>
+    <t>word_confidence_mean</t>
+  </si>
+  <si>
+    <t>word_confidence_sd</t>
+  </si>
+  <si>
+    <t>etters</t>
+  </si>
+  <si>
+    <t>syllables</t>
   </si>
 </sst>
 </file>
@@ -1666,7 +1936,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
-    <numFmt numFmtId="166" formatCode="0.00000000"/>
+    <numFmt numFmtId="164" formatCode="0.00000000"/>
   </numFmts>
   <fonts count="6" x14ac:knownFonts="1">
     <font>
@@ -1760,21 +2030,21 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="right" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment horizontal="right" wrapText="1"/>
-    </xf>
-    <xf numFmtId="166" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normale" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
@@ -2075,798 +2345,6 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1E213513-60BC-A545-BBC0-EED3A764549D}">
-  <dimension ref="A1:D105"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="14" x14ac:dyDescent="0.2"/>
-  <cols>
-    <col min="1" max="1" width="18.5" style="10" customWidth="1"/>
-    <col min="2" max="2" width="137.33203125" style="2" bestFit="1" customWidth="1"/>
-    <col min="3" max="16384" width="8.6640625" style="2"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A1" s="11" t="s">
-        <v>451</v>
-      </c>
-      <c r="B1" s="11"/>
-    </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A3" s="3"/>
-      <c r="B3" s="4"/>
-    </row>
-    <row r="4" spans="1:2" ht="15" x14ac:dyDescent="0.2">
-      <c r="A4" s="3" t="s">
-        <v>0</v>
-      </c>
-      <c r="B4" s="5" t="s">
-        <v>543</v>
-      </c>
-    </row>
-    <row r="5" spans="1:2" ht="15" x14ac:dyDescent="0.2">
-      <c r="A5" s="3" t="s">
-        <v>1</v>
-      </c>
-      <c r="B5" s="4" t="s">
-        <v>452</v>
-      </c>
-    </row>
-    <row r="6" spans="1:2" ht="15" x14ac:dyDescent="0.2">
-      <c r="A6" s="3" t="s">
-        <v>2</v>
-      </c>
-      <c r="B6" s="4" t="s">
-        <v>453</v>
-      </c>
-    </row>
-    <row r="7" spans="1:2" ht="15" x14ac:dyDescent="0.2">
-      <c r="A7" s="3" t="s">
-        <v>3</v>
-      </c>
-      <c r="B7" s="4" t="s">
-        <v>454</v>
-      </c>
-    </row>
-    <row r="8" spans="1:2" ht="15" x14ac:dyDescent="0.2">
-      <c r="A8" s="3" t="s">
-        <v>4</v>
-      </c>
-      <c r="B8" s="4" t="s">
-        <v>455</v>
-      </c>
-    </row>
-    <row r="9" spans="1:2" ht="15" x14ac:dyDescent="0.2">
-      <c r="A9" s="6" t="s">
-        <v>5</v>
-      </c>
-      <c r="B9" s="4" t="s">
-        <v>456</v>
-      </c>
-    </row>
-    <row r="10" spans="1:2" ht="15" x14ac:dyDescent="0.2">
-      <c r="A10" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="B10" s="4" t="s">
-        <v>457</v>
-      </c>
-    </row>
-    <row r="11" spans="1:2" ht="15" x14ac:dyDescent="0.2">
-      <c r="A11" s="6" t="s">
-        <v>7</v>
-      </c>
-      <c r="B11" s="4" t="s">
-        <v>458</v>
-      </c>
-    </row>
-    <row r="12" spans="1:2" ht="15" x14ac:dyDescent="0.2">
-      <c r="A12" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="B12" s="4" t="s">
-        <v>459</v>
-      </c>
-    </row>
-    <row r="13" spans="1:2" ht="15" x14ac:dyDescent="0.2">
-      <c r="A13" s="6" t="s">
-        <v>9</v>
-      </c>
-      <c r="B13" s="4" t="s">
-        <v>460</v>
-      </c>
-    </row>
-    <row r="14" spans="1:2" ht="15" x14ac:dyDescent="0.2">
-      <c r="A14" s="6" t="s">
-        <v>10</v>
-      </c>
-      <c r="B14" s="4" t="s">
-        <v>461</v>
-      </c>
-    </row>
-    <row r="15" spans="1:2" ht="15" x14ac:dyDescent="0.2">
-      <c r="A15" s="6" t="s">
-        <v>11</v>
-      </c>
-      <c r="B15" s="7" t="s">
-        <v>458</v>
-      </c>
-    </row>
-    <row r="16" spans="1:2" ht="15" x14ac:dyDescent="0.2">
-      <c r="A16" s="6" t="s">
-        <v>12</v>
-      </c>
-      <c r="B16" s="4" t="s">
-        <v>462</v>
-      </c>
-    </row>
-    <row r="17" spans="1:2" ht="15" x14ac:dyDescent="0.2">
-      <c r="A17" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="B17" s="7" t="s">
-        <v>463</v>
-      </c>
-    </row>
-    <row r="18" spans="1:2" ht="15" x14ac:dyDescent="0.2">
-      <c r="A18" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="B18" s="7" t="s">
-        <v>464</v>
-      </c>
-    </row>
-    <row r="19" spans="1:2" ht="15" x14ac:dyDescent="0.2">
-      <c r="A19" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="B19" s="4" t="s">
-        <v>465</v>
-      </c>
-    </row>
-    <row r="20" spans="1:2" ht="15" x14ac:dyDescent="0.2">
-      <c r="A20" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="B20" s="4" t="s">
-        <v>466</v>
-      </c>
-    </row>
-    <row r="21" spans="1:2" ht="15" x14ac:dyDescent="0.2">
-      <c r="A21" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="B21" s="4" t="s">
-        <v>467</v>
-      </c>
-    </row>
-    <row r="22" spans="1:2" ht="15" x14ac:dyDescent="0.2">
-      <c r="A22" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="B22" s="4" t="s">
-        <v>468</v>
-      </c>
-    </row>
-    <row r="23" spans="1:2" ht="15" x14ac:dyDescent="0.2">
-      <c r="A23" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="B23" s="4" t="s">
-        <v>469</v>
-      </c>
-    </row>
-    <row r="24" spans="1:2" ht="15" x14ac:dyDescent="0.2">
-      <c r="A24" s="3" t="s">
-        <v>20</v>
-      </c>
-      <c r="B24" s="4" t="s">
-        <v>470</v>
-      </c>
-    </row>
-    <row r="25" spans="1:2" ht="15" x14ac:dyDescent="0.2">
-      <c r="A25" s="3" t="s">
-        <v>21</v>
-      </c>
-      <c r="B25" s="4" t="s">
-        <v>471</v>
-      </c>
-    </row>
-    <row r="26" spans="1:2" ht="15" x14ac:dyDescent="0.2">
-      <c r="A26" s="3" t="s">
-        <v>22</v>
-      </c>
-      <c r="B26" s="4" t="s">
-        <v>472</v>
-      </c>
-    </row>
-    <row r="27" spans="1:2" ht="15" x14ac:dyDescent="0.2">
-      <c r="A27" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="B27" s="4" t="s">
-        <v>473</v>
-      </c>
-    </row>
-    <row r="28" spans="1:2" ht="15" x14ac:dyDescent="0.2">
-      <c r="A28" s="3" t="s">
-        <v>24</v>
-      </c>
-      <c r="B28" s="4" t="s">
-        <v>474</v>
-      </c>
-    </row>
-    <row r="29" spans="1:2" ht="15" x14ac:dyDescent="0.2">
-      <c r="A29" s="3" t="s">
-        <v>31</v>
-      </c>
-      <c r="B29" s="4" t="s">
-        <v>475</v>
-      </c>
-    </row>
-    <row r="30" spans="1:2" ht="15" x14ac:dyDescent="0.2">
-      <c r="A30" s="3" t="s">
-        <v>32</v>
-      </c>
-      <c r="B30" s="4" t="s">
-        <v>476</v>
-      </c>
-    </row>
-    <row r="31" spans="1:2" ht="15" x14ac:dyDescent="0.2">
-      <c r="A31" s="3" t="s">
-        <v>25</v>
-      </c>
-      <c r="B31" s="4" t="s">
-        <v>477</v>
-      </c>
-    </row>
-    <row r="32" spans="1:2" ht="15" x14ac:dyDescent="0.2">
-      <c r="A32" s="3" t="s">
-        <v>26</v>
-      </c>
-      <c r="B32" s="4" t="s">
-        <v>478</v>
-      </c>
-    </row>
-    <row r="33" spans="1:2" ht="15" x14ac:dyDescent="0.2">
-      <c r="A33" s="3" t="s">
-        <v>27</v>
-      </c>
-      <c r="B33" s="4" t="s">
-        <v>479</v>
-      </c>
-    </row>
-    <row r="34" spans="1:2" ht="15" x14ac:dyDescent="0.2">
-      <c r="A34" s="3" t="s">
-        <v>28</v>
-      </c>
-      <c r="B34" s="4" t="s">
-        <v>480</v>
-      </c>
-    </row>
-    <row r="35" spans="1:2" ht="15" x14ac:dyDescent="0.2">
-      <c r="A35" s="3" t="s">
-        <v>29</v>
-      </c>
-      <c r="B35" s="4" t="s">
-        <v>481</v>
-      </c>
-    </row>
-    <row r="36" spans="1:2" ht="15" x14ac:dyDescent="0.2">
-      <c r="A36" s="3" t="s">
-        <v>30</v>
-      </c>
-      <c r="B36" s="4" t="s">
-        <v>482</v>
-      </c>
-    </row>
-    <row r="37" spans="1:2" ht="15" x14ac:dyDescent="0.2">
-      <c r="A37" s="3" t="s">
-        <v>536</v>
-      </c>
-      <c r="B37" s="4" t="s">
-        <v>538</v>
-      </c>
-    </row>
-    <row r="38" spans="1:2" ht="15" x14ac:dyDescent="0.2">
-      <c r="A38" s="3" t="s">
-        <v>537</v>
-      </c>
-      <c r="B38" s="4" t="s">
-        <v>539</v>
-      </c>
-    </row>
-    <row r="39" spans="1:2" ht="15" x14ac:dyDescent="0.2">
-      <c r="A39" s="3" t="s">
-        <v>33</v>
-      </c>
-      <c r="B39" s="4" t="s">
-        <v>483</v>
-      </c>
-    </row>
-    <row r="40" spans="1:2" ht="15" x14ac:dyDescent="0.2">
-      <c r="A40" s="3" t="s">
-        <v>34</v>
-      </c>
-      <c r="B40" s="4" t="s">
-        <v>484</v>
-      </c>
-    </row>
-    <row r="41" spans="1:2" ht="15" x14ac:dyDescent="0.2">
-      <c r="A41" s="3" t="s">
-        <v>541</v>
-      </c>
-      <c r="B41" s="4" t="s">
-        <v>545</v>
-      </c>
-    </row>
-    <row r="42" spans="1:2" ht="15" x14ac:dyDescent="0.2">
-      <c r="A42" s="3" t="s">
-        <v>542</v>
-      </c>
-      <c r="B42" s="4" t="s">
-        <v>485</v>
-      </c>
-    </row>
-    <row r="43" spans="1:2" ht="15" x14ac:dyDescent="0.2">
-      <c r="A43" s="3" t="s">
-        <v>540</v>
-      </c>
-      <c r="B43" s="4" t="s">
-        <v>544</v>
-      </c>
-    </row>
-    <row r="44" spans="1:2" ht="15" x14ac:dyDescent="0.2">
-      <c r="A44" s="3" t="s">
-        <v>35</v>
-      </c>
-      <c r="B44" s="4" t="s">
-        <v>486</v>
-      </c>
-    </row>
-    <row r="45" spans="1:2" ht="15" x14ac:dyDescent="0.2">
-      <c r="A45" s="3" t="s">
-        <v>36</v>
-      </c>
-      <c r="B45" s="4" t="s">
-        <v>487</v>
-      </c>
-    </row>
-    <row r="46" spans="1:2" ht="15" x14ac:dyDescent="0.2">
-      <c r="A46" s="3" t="s">
-        <v>37</v>
-      </c>
-      <c r="B46" s="4" t="s">
-        <v>488</v>
-      </c>
-    </row>
-    <row r="47" spans="1:2" ht="15" x14ac:dyDescent="0.2">
-      <c r="A47" s="3" t="s">
-        <v>38</v>
-      </c>
-      <c r="B47" s="4" t="s">
-        <v>489</v>
-      </c>
-    </row>
-    <row r="48" spans="1:2" ht="15" x14ac:dyDescent="0.2">
-      <c r="A48" s="3" t="s">
-        <v>39</v>
-      </c>
-      <c r="B48" s="4" t="s">
-        <v>490</v>
-      </c>
-    </row>
-    <row r="49" spans="1:2" ht="15" x14ac:dyDescent="0.2">
-      <c r="A49" s="3" t="s">
-        <v>40</v>
-      </c>
-      <c r="B49" s="4" t="s">
-        <v>491</v>
-      </c>
-    </row>
-    <row r="50" spans="1:2" ht="15" x14ac:dyDescent="0.2">
-      <c r="A50" s="3" t="s">
-        <v>37</v>
-      </c>
-      <c r="B50" s="4" t="s">
-        <v>488</v>
-      </c>
-    </row>
-    <row r="51" spans="1:2" ht="15" x14ac:dyDescent="0.2">
-      <c r="A51" s="3" t="s">
-        <v>38</v>
-      </c>
-      <c r="B51" s="4" t="s">
-        <v>489</v>
-      </c>
-    </row>
-    <row r="52" spans="1:2" ht="15" x14ac:dyDescent="0.2">
-      <c r="A52" s="3" t="s">
-        <v>41</v>
-      </c>
-      <c r="B52" s="4" t="s">
-        <v>492</v>
-      </c>
-    </row>
-    <row r="53" spans="1:2" ht="15" x14ac:dyDescent="0.2">
-      <c r="A53" s="3" t="s">
-        <v>42</v>
-      </c>
-      <c r="B53" s="4" t="s">
-        <v>493</v>
-      </c>
-    </row>
-    <row r="54" spans="1:2" ht="15" x14ac:dyDescent="0.2">
-      <c r="A54" s="3" t="s">
-        <v>41</v>
-      </c>
-      <c r="B54" s="4" t="s">
-        <v>492</v>
-      </c>
-    </row>
-    <row r="55" spans="1:2" ht="15" x14ac:dyDescent="0.2">
-      <c r="A55" s="3" t="s">
-        <v>42</v>
-      </c>
-      <c r="B55" s="4" t="s">
-        <v>493</v>
-      </c>
-    </row>
-    <row r="56" spans="1:2" ht="15" x14ac:dyDescent="0.2">
-      <c r="A56" s="3" t="s">
-        <v>43</v>
-      </c>
-      <c r="B56" s="4" t="s">
-        <v>494</v>
-      </c>
-    </row>
-    <row r="57" spans="1:2" ht="15" x14ac:dyDescent="0.2">
-      <c r="A57" s="3" t="s">
-        <v>44</v>
-      </c>
-      <c r="B57" s="4" t="s">
-        <v>495</v>
-      </c>
-    </row>
-    <row r="58" spans="1:2" ht="15" x14ac:dyDescent="0.2">
-      <c r="A58" s="3" t="s">
-        <v>45</v>
-      </c>
-      <c r="B58" s="4" t="s">
-        <v>496</v>
-      </c>
-    </row>
-    <row r="59" spans="1:2" ht="15" x14ac:dyDescent="0.2">
-      <c r="A59" s="3" t="s">
-        <v>46</v>
-      </c>
-      <c r="B59" s="4" t="s">
-        <v>497</v>
-      </c>
-    </row>
-    <row r="60" spans="1:2" ht="15" x14ac:dyDescent="0.2">
-      <c r="A60" s="3" t="s">
-        <v>47</v>
-      </c>
-      <c r="B60" s="4" t="s">
-        <v>498</v>
-      </c>
-    </row>
-    <row r="61" spans="1:2" ht="15" x14ac:dyDescent="0.2">
-      <c r="A61" s="3" t="s">
-        <v>48</v>
-      </c>
-      <c r="B61" s="4" t="s">
-        <v>499</v>
-      </c>
-    </row>
-    <row r="62" spans="1:2" ht="15" x14ac:dyDescent="0.2">
-      <c r="A62" s="3" t="s">
-        <v>49</v>
-      </c>
-      <c r="B62" s="4" t="s">
-        <v>500</v>
-      </c>
-    </row>
-    <row r="63" spans="1:2" ht="15" x14ac:dyDescent="0.2">
-      <c r="A63" s="3" t="s">
-        <v>50</v>
-      </c>
-      <c r="B63" s="4" t="s">
-        <v>501</v>
-      </c>
-    </row>
-    <row r="64" spans="1:2" ht="15" x14ac:dyDescent="0.2">
-      <c r="A64" s="3" t="s">
-        <v>51</v>
-      </c>
-      <c r="B64" s="4" t="s">
-        <v>502</v>
-      </c>
-    </row>
-    <row r="65" spans="1:2" ht="15" x14ac:dyDescent="0.2">
-      <c r="A65" s="3" t="s">
-        <v>52</v>
-      </c>
-      <c r="B65" s="4" t="s">
-        <v>503</v>
-      </c>
-    </row>
-    <row r="66" spans="1:2" ht="15" x14ac:dyDescent="0.2">
-      <c r="A66" s="3" t="s">
-        <v>55</v>
-      </c>
-      <c r="B66" s="4" t="s">
-        <v>504</v>
-      </c>
-    </row>
-    <row r="67" spans="1:2" ht="15" x14ac:dyDescent="0.2">
-      <c r="A67" s="3" t="s">
-        <v>56</v>
-      </c>
-      <c r="B67" s="4" t="s">
-        <v>505</v>
-      </c>
-    </row>
-    <row r="68" spans="1:2" ht="15" x14ac:dyDescent="0.2">
-      <c r="A68" s="3" t="s">
-        <v>57</v>
-      </c>
-      <c r="B68" s="4" t="s">
-        <v>506</v>
-      </c>
-    </row>
-    <row r="69" spans="1:2" ht="15" x14ac:dyDescent="0.2">
-      <c r="A69" s="3" t="s">
-        <v>58</v>
-      </c>
-      <c r="B69" s="4" t="s">
-        <v>507</v>
-      </c>
-    </row>
-    <row r="70" spans="1:2" ht="15" x14ac:dyDescent="0.2">
-      <c r="A70" s="3" t="s">
-        <v>53</v>
-      </c>
-      <c r="B70" s="4" t="s">
-        <v>508</v>
-      </c>
-    </row>
-    <row r="71" spans="1:2" ht="15" x14ac:dyDescent="0.2">
-      <c r="A71" s="3" t="s">
-        <v>54</v>
-      </c>
-      <c r="B71" s="4" t="s">
-        <v>509</v>
-      </c>
-    </row>
-    <row r="72" spans="1:2" ht="15" x14ac:dyDescent="0.2">
-      <c r="A72" s="3" t="s">
-        <v>61</v>
-      </c>
-      <c r="B72" s="4" t="s">
-        <v>510</v>
-      </c>
-    </row>
-    <row r="73" spans="1:2" ht="15" x14ac:dyDescent="0.2">
-      <c r="A73" s="3" t="s">
-        <v>62</v>
-      </c>
-      <c r="B73" s="4" t="s">
-        <v>511</v>
-      </c>
-    </row>
-    <row r="74" spans="1:2" ht="15" x14ac:dyDescent="0.2">
-      <c r="A74" s="3" t="s">
-        <v>71</v>
-      </c>
-      <c r="B74" s="4" t="s">
-        <v>512</v>
-      </c>
-    </row>
-    <row r="75" spans="1:2" ht="15" x14ac:dyDescent="0.2">
-      <c r="A75" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="B75" s="4" t="s">
-        <v>513</v>
-      </c>
-    </row>
-    <row r="76" spans="1:2" ht="15" x14ac:dyDescent="0.2">
-      <c r="A76" s="3" t="s">
-        <v>69</v>
-      </c>
-      <c r="B76" s="4" t="s">
-        <v>514</v>
-      </c>
-    </row>
-    <row r="77" spans="1:2" ht="15" x14ac:dyDescent="0.2">
-      <c r="A77" s="3" t="s">
-        <v>70</v>
-      </c>
-      <c r="B77" s="4" t="s">
-        <v>515</v>
-      </c>
-    </row>
-    <row r="78" spans="1:2" ht="15" x14ac:dyDescent="0.2">
-      <c r="A78" s="3" t="s">
-        <v>63</v>
-      </c>
-      <c r="B78" s="4" t="s">
-        <v>516</v>
-      </c>
-    </row>
-    <row r="79" spans="1:2" ht="15" x14ac:dyDescent="0.2">
-      <c r="A79" s="3" t="s">
-        <v>64</v>
-      </c>
-      <c r="B79" s="4" t="s">
-        <v>517</v>
-      </c>
-    </row>
-    <row r="80" spans="1:2" ht="15" x14ac:dyDescent="0.2">
-      <c r="A80" s="3" t="s">
-        <v>67</v>
-      </c>
-      <c r="B80" s="4" t="s">
-        <v>518</v>
-      </c>
-    </row>
-    <row r="81" spans="1:4" ht="15" x14ac:dyDescent="0.2">
-      <c r="A81" s="3" t="s">
-        <v>68</v>
-      </c>
-      <c r="B81" s="4" t="s">
-        <v>519</v>
-      </c>
-    </row>
-    <row r="82" spans="1:4" ht="15" x14ac:dyDescent="0.2">
-      <c r="A82" s="3" t="s">
-        <v>65</v>
-      </c>
-      <c r="B82" s="4" t="s">
-        <v>520</v>
-      </c>
-    </row>
-    <row r="83" spans="1:4" ht="15" x14ac:dyDescent="0.2">
-      <c r="A83" s="3" t="s">
-        <v>66</v>
-      </c>
-      <c r="B83" s="4" t="s">
-        <v>521</v>
-      </c>
-    </row>
-    <row r="84" spans="1:4" ht="15" x14ac:dyDescent="0.2">
-      <c r="A84" s="3" t="s">
-        <v>59</v>
-      </c>
-      <c r="B84" s="4" t="s">
-        <v>522</v>
-      </c>
-    </row>
-    <row r="85" spans="1:4" ht="15" x14ac:dyDescent="0.2">
-      <c r="A85" s="3" t="s">
-        <v>60</v>
-      </c>
-      <c r="B85" s="4" t="s">
-        <v>523</v>
-      </c>
-    </row>
-    <row r="86" spans="1:4" ht="15" x14ac:dyDescent="0.2">
-      <c r="A86" s="3" t="s">
-        <v>73</v>
-      </c>
-      <c r="B86" s="4" t="s">
-        <v>524</v>
-      </c>
-    </row>
-    <row r="87" spans="1:4" ht="15" x14ac:dyDescent="0.2">
-      <c r="A87" s="3" t="s">
-        <v>74</v>
-      </c>
-      <c r="B87" s="4" t="s">
-        <v>525</v>
-      </c>
-    </row>
-    <row r="88" spans="1:4" ht="15" x14ac:dyDescent="0.2">
-      <c r="A88" s="3" t="s">
-        <v>75</v>
-      </c>
-      <c r="B88" s="4" t="s">
-        <v>526</v>
-      </c>
-    </row>
-    <row r="89" spans="1:4" ht="15" x14ac:dyDescent="0.2">
-      <c r="A89" s="3" t="s">
-        <v>76</v>
-      </c>
-      <c r="B89" s="4" t="s">
-        <v>527</v>
-      </c>
-    </row>
-    <row r="90" spans="1:4" ht="15" x14ac:dyDescent="0.2">
-      <c r="A90" s="3" t="s">
-        <v>77</v>
-      </c>
-      <c r="B90" s="4" t="s">
-        <v>528</v>
-      </c>
-    </row>
-    <row r="91" spans="1:4" ht="15" x14ac:dyDescent="0.2">
-      <c r="A91" s="3" t="s">
-        <v>78</v>
-      </c>
-      <c r="B91" s="4" t="s">
-        <v>529</v>
-      </c>
-    </row>
-    <row r="92" spans="1:4" ht="15" x14ac:dyDescent="0.2">
-      <c r="A92" s="3" t="s">
-        <v>79</v>
-      </c>
-      <c r="B92" s="4" t="s">
-        <v>530</v>
-      </c>
-    </row>
-    <row r="93" spans="1:4" ht="15" x14ac:dyDescent="0.2">
-      <c r="A93" s="3" t="s">
-        <v>80</v>
-      </c>
-      <c r="B93" s="4" t="s">
-        <v>531</v>
-      </c>
-    </row>
-    <row r="94" spans="1:4" ht="15" x14ac:dyDescent="0.2">
-      <c r="A94" s="3" t="s">
-        <v>81</v>
-      </c>
-      <c r="B94" s="4" t="s">
-        <v>532</v>
-      </c>
-    </row>
-    <row r="95" spans="1:4" ht="15" x14ac:dyDescent="0.2">
-      <c r="A95" s="3" t="s">
-        <v>82</v>
-      </c>
-      <c r="B95" s="4" t="s">
-        <v>533</v>
-      </c>
-    </row>
-    <row r="96" spans="1:4" ht="15" x14ac:dyDescent="0.2">
-      <c r="A96" s="8" t="s">
-        <v>83</v>
-      </c>
-      <c r="B96" s="5" t="s">
-        <v>534</v>
-      </c>
-      <c r="C96" s="1"/>
-      <c r="D96" s="1"/>
-    </row>
-    <row r="97" spans="1:4" ht="15" x14ac:dyDescent="0.2">
-      <c r="A97" s="9" t="s">
-        <v>84</v>
-      </c>
-      <c r="B97" s="5" t="s">
-        <v>535</v>
-      </c>
-      <c r="C97" s="1"/>
-      <c r="D97" s="1"/>
-    </row>
-    <row r="104" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A104" s="3"/>
-      <c r="B104" s="4"/>
-    </row>
-    <row r="105" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A105" s="3"/>
-      <c r="B105" s="4"/>
-    </row>
-  </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="A1:B1"/>
-  </mergeCells>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:CL201"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
@@ -2910,7 +2388,7 @@
     <col min="37" max="37" width="7.33203125" bestFit="1" customWidth="1"/>
     <col min="38" max="38" width="11" bestFit="1" customWidth="1"/>
     <col min="39" max="39" width="11.1640625" bestFit="1" customWidth="1"/>
-    <col min="40" max="40" width="10.6640625" style="12" bestFit="1" customWidth="1"/>
+    <col min="40" max="40" width="10.6640625" style="11" bestFit="1" customWidth="1"/>
     <col min="41" max="41" width="6.83203125" bestFit="1" customWidth="1"/>
     <col min="42" max="42" width="7" bestFit="1" customWidth="1"/>
     <col min="43" max="43" width="6" bestFit="1" customWidth="1"/>
@@ -2962,274 +2440,274 @@
   <sheetData>
     <row r="1" spans="1:90" s="1" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
-        <v>0</v>
+        <v>546</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>1</v>
+        <v>547</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>3</v>
+        <v>548</v>
+      </c>
+      <c r="D1" t="s">
+        <v>549</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>4</v>
+        <v>550</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>5</v>
+        <v>551</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>6</v>
+        <v>552</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>7</v>
+        <v>553</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>8</v>
+        <v>554</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>9</v>
+        <v>555</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>10</v>
+        <v>556</v>
       </c>
       <c r="L1" s="1" t="s">
-        <v>11</v>
+        <v>557</v>
       </c>
       <c r="M1" s="1" t="s">
-        <v>12</v>
+        <v>558</v>
       </c>
       <c r="N1" s="1" t="s">
-        <v>13</v>
+        <v>559</v>
       </c>
       <c r="O1" s="1" t="s">
-        <v>14</v>
+        <v>560</v>
       </c>
       <c r="P1" s="1" t="s">
-        <v>15</v>
+        <v>561</v>
       </c>
       <c r="Q1" s="1" t="s">
-        <v>16</v>
+        <v>562</v>
       </c>
       <c r="R1" s="1" t="s">
-        <v>17</v>
+        <v>563</v>
       </c>
       <c r="S1" s="1" t="s">
-        <v>18</v>
+        <v>564</v>
       </c>
       <c r="T1" s="1" t="s">
-        <v>19</v>
+        <v>565</v>
       </c>
       <c r="U1" s="1" t="s">
-        <v>20</v>
+        <v>566</v>
       </c>
       <c r="V1" s="1" t="s">
-        <v>21</v>
+        <v>567</v>
       </c>
       <c r="W1" s="1" t="s">
-        <v>22</v>
+        <v>568</v>
       </c>
       <c r="X1" s="1" t="s">
-        <v>23</v>
+        <v>569</v>
       </c>
       <c r="Y1" s="1" t="s">
-        <v>24</v>
+        <v>570</v>
       </c>
       <c r="Z1" s="1" t="s">
-        <v>25</v>
+        <v>571</v>
       </c>
       <c r="AA1" s="1" t="s">
-        <v>26</v>
+        <v>572</v>
       </c>
       <c r="AB1" s="1" t="s">
-        <v>27</v>
+        <v>573</v>
       </c>
       <c r="AC1" s="1" t="s">
-        <v>28</v>
+        <v>574</v>
       </c>
       <c r="AD1" s="1" t="s">
-        <v>29</v>
+        <v>575</v>
       </c>
       <c r="AE1" s="1" t="s">
-        <v>30</v>
+        <v>576</v>
       </c>
       <c r="AF1" s="1" t="s">
-        <v>536</v>
+        <v>577</v>
       </c>
       <c r="AG1" s="1" t="s">
-        <v>537</v>
+        <v>578</v>
       </c>
       <c r="AH1" s="1" t="s">
-        <v>31</v>
+        <v>579</v>
       </c>
       <c r="AI1" s="1" t="s">
-        <v>32</v>
+        <v>580</v>
       </c>
       <c r="AJ1" s="1" t="s">
-        <v>33</v>
+        <v>581</v>
       </c>
       <c r="AK1" s="1" t="s">
-        <v>34</v>
+        <v>582</v>
       </c>
       <c r="AL1" s="1" t="s">
-        <v>541</v>
+        <v>583</v>
       </c>
       <c r="AM1" s="1" t="s">
-        <v>542</v>
-      </c>
-      <c r="AN1" s="14" t="s">
-        <v>540</v>
+        <v>584</v>
+      </c>
+      <c r="AN1" s="13" t="s">
+        <v>585</v>
       </c>
       <c r="AO1" s="1" t="s">
-        <v>35</v>
+        <v>586</v>
       </c>
       <c r="AP1" s="1" t="s">
-        <v>36</v>
+        <v>587</v>
       </c>
       <c r="AQ1" s="1" t="s">
-        <v>37</v>
+        <v>588</v>
       </c>
       <c r="AR1" s="1" t="s">
-        <v>38</v>
+        <v>589</v>
       </c>
       <c r="AS1" s="1" t="s">
-        <v>39</v>
+        <v>590</v>
       </c>
       <c r="AT1" s="1" t="s">
-        <v>40</v>
+        <v>591</v>
       </c>
       <c r="AU1" s="1" t="s">
-        <v>41</v>
+        <v>592</v>
       </c>
       <c r="AV1" s="1" t="s">
-        <v>42</v>
+        <v>593</v>
       </c>
       <c r="AW1" s="1" t="s">
-        <v>43</v>
+        <v>594</v>
       </c>
       <c r="AX1" s="1" t="s">
-        <v>44</v>
+        <v>595</v>
       </c>
       <c r="AY1" s="1" t="s">
-        <v>45</v>
+        <v>596</v>
       </c>
       <c r="AZ1" s="1" t="s">
-        <v>46</v>
+        <v>597</v>
       </c>
       <c r="BA1" s="1" t="s">
-        <v>47</v>
+        <v>598</v>
       </c>
       <c r="BB1" s="1" t="s">
-        <v>48</v>
+        <v>599</v>
       </c>
       <c r="BC1" s="1" t="s">
-        <v>49</v>
+        <v>600</v>
       </c>
       <c r="BD1" s="1" t="s">
-        <v>50</v>
+        <v>601</v>
       </c>
       <c r="BE1" s="1" t="s">
-        <v>51</v>
+        <v>602</v>
       </c>
       <c r="BF1" s="1" t="s">
-        <v>52</v>
+        <v>603</v>
       </c>
       <c r="BG1" s="1" t="s">
-        <v>53</v>
+        <v>604</v>
       </c>
       <c r="BH1" s="1" t="s">
-        <v>54</v>
+        <v>605</v>
       </c>
       <c r="BI1" s="1" t="s">
-        <v>55</v>
+        <v>606</v>
       </c>
       <c r="BJ1" s="1" t="s">
-        <v>56</v>
+        <v>607</v>
       </c>
       <c r="BK1" s="1" t="s">
-        <v>57</v>
+        <v>608</v>
       </c>
       <c r="BL1" s="1" t="s">
-        <v>58</v>
+        <v>609</v>
       </c>
       <c r="BM1" s="1" t="s">
-        <v>59</v>
+        <v>610</v>
       </c>
       <c r="BN1" s="1" t="s">
-        <v>60</v>
+        <v>611</v>
       </c>
       <c r="BO1" s="1" t="s">
-        <v>61</v>
+        <v>612</v>
       </c>
       <c r="BP1" s="1" t="s">
-        <v>62</v>
+        <v>613</v>
       </c>
       <c r="BQ1" s="1" t="s">
-        <v>63</v>
+        <v>614</v>
       </c>
       <c r="BR1" s="1" t="s">
-        <v>64</v>
+        <v>615</v>
       </c>
       <c r="BS1" s="1" t="s">
-        <v>65</v>
+        <v>616</v>
       </c>
       <c r="BT1" s="1" t="s">
-        <v>66</v>
+        <v>617</v>
       </c>
       <c r="BU1" s="1" t="s">
-        <v>67</v>
+        <v>618</v>
       </c>
       <c r="BV1" s="1" t="s">
-        <v>68</v>
+        <v>619</v>
       </c>
       <c r="BW1" s="1" t="s">
-        <v>69</v>
+        <v>620</v>
       </c>
       <c r="BX1" s="1" t="s">
-        <v>70</v>
+        <v>621</v>
       </c>
       <c r="BY1" s="1" t="s">
-        <v>71</v>
+        <v>622</v>
       </c>
       <c r="BZ1" s="1" t="s">
-        <v>72</v>
+        <v>623</v>
       </c>
       <c r="CA1" s="1" t="s">
-        <v>73</v>
+        <v>624</v>
       </c>
       <c r="CB1" s="1" t="s">
-        <v>74</v>
+        <v>625</v>
       </c>
       <c r="CC1" s="1" t="s">
-        <v>75</v>
+        <v>626</v>
       </c>
       <c r="CD1" s="1" t="s">
-        <v>76</v>
+        <v>627</v>
       </c>
       <c r="CE1" s="1" t="s">
-        <v>77</v>
+        <v>628</v>
       </c>
       <c r="CF1" s="1" t="s">
-        <v>78</v>
+        <v>629</v>
       </c>
       <c r="CG1" s="1" t="s">
-        <v>79</v>
+        <v>630</v>
       </c>
       <c r="CH1" s="1" t="s">
-        <v>80</v>
+        <v>631</v>
       </c>
       <c r="CI1" s="1" t="s">
-        <v>81</v>
+        <v>632</v>
       </c>
       <c r="CJ1" s="1" t="s">
-        <v>82</v>
+        <v>633</v>
       </c>
       <c r="CK1" s="1" t="s">
-        <v>83</v>
+        <v>634</v>
       </c>
       <c r="CL1" s="1" t="s">
-        <v>84</v>
+        <v>635</v>
       </c>
     </row>
     <row r="2" spans="1:90" x14ac:dyDescent="0.2">
@@ -3350,7 +2828,7 @@
       <c r="AM2">
         <v>1.28</v>
       </c>
-      <c r="AN2" s="12">
+      <c r="AN2" s="11">
         <v>2.5971000000000001E-6</v>
       </c>
       <c r="AO2">
@@ -3622,7 +3100,7 @@
       <c r="AM3">
         <v>1.26</v>
       </c>
-      <c r="AN3" s="12">
+      <c r="AN3" s="11">
         <v>2.4930999999999999E-6</v>
       </c>
       <c r="AO3">
@@ -3894,7 +3372,7 @@
       <c r="AM4">
         <v>1.25</v>
       </c>
-      <c r="AN4" s="12">
+      <c r="AN4" s="11">
         <v>4.6446999999999998E-6</v>
       </c>
       <c r="AO4">
@@ -4166,7 +3644,7 @@
       <c r="AM5">
         <v>1.34</v>
       </c>
-      <c r="AN5" s="12">
+      <c r="AN5" s="11">
         <v>6.9670000000000004E-6</v>
       </c>
       <c r="AO5">
@@ -4438,7 +3916,7 @@
       <c r="AM6">
         <v>1.1399999999999999</v>
       </c>
-      <c r="AN6" s="12">
+      <c r="AN6" s="11">
         <v>5.3424394999999998E-3</v>
       </c>
       <c r="AO6">
@@ -4710,7 +4188,7 @@
       <c r="AM7">
         <v>1.24</v>
       </c>
-      <c r="AN7" s="12">
+      <c r="AN7" s="11">
         <v>1.9146359999999999E-4</v>
       </c>
       <c r="AO7">
@@ -4982,7 +4460,7 @@
       <c r="AM8">
         <v>1</v>
       </c>
-      <c r="AN8" s="12">
+      <c r="AN8" s="11">
         <v>5.7375999999999999E-6</v>
       </c>
       <c r="AO8">
@@ -5254,7 +4732,7 @@
       <c r="AM9">
         <v>1.43</v>
       </c>
-      <c r="AN9" s="12">
+      <c r="AN9" s="11">
         <v>1.9152509999999999E-4</v>
       </c>
       <c r="AO9">
@@ -5526,7 +5004,7 @@
       <c r="AM10">
         <v>1.1499999999999999</v>
       </c>
-      <c r="AN10" s="12">
+      <c r="AN10" s="11">
         <v>6.9670000000000004E-6</v>
       </c>
       <c r="AO10">
@@ -5798,7 +5276,7 @@
       <c r="AM11">
         <v>1.1499999999999999</v>
       </c>
-      <c r="AN11" s="12">
+      <c r="AN11" s="11">
         <v>2.3892546000000001E-3</v>
       </c>
       <c r="AO11">
@@ -6070,7 +5548,7 @@
       <c r="AM12">
         <v>1.53</v>
       </c>
-      <c r="AN12" s="12">
+      <c r="AN12" s="11">
         <v>4.0399199999999998E-5</v>
       </c>
       <c r="AO12">
@@ -6342,7 +5820,7 @@
       <c r="AM13">
         <v>1.52</v>
       </c>
-      <c r="AN13" s="12">
+      <c r="AN13" s="11">
         <v>9.2124699999999996E-5</v>
       </c>
       <c r="AO13">
@@ -6614,7 +6092,7 @@
       <c r="AM14">
         <v>1.21</v>
       </c>
-      <c r="AN14" s="12">
+      <c r="AN14" s="11">
         <v>7.8100000000000005E-8</v>
       </c>
       <c r="AO14">
@@ -6886,7 +6364,7 @@
       <c r="AM15">
         <v>1.29</v>
       </c>
-      <c r="AN15" s="12">
+      <c r="AN15" s="11">
         <v>4.1460700000000001E-5</v>
       </c>
       <c r="AO15">
@@ -7158,7 +6636,7 @@
       <c r="AM16">
         <v>1.52</v>
       </c>
-      <c r="AN16" s="12">
+      <c r="AN16" s="11">
         <v>4.5160600000000003E-5</v>
       </c>
       <c r="AO16">
@@ -7430,7 +6908,7 @@
       <c r="AM17">
         <v>1.1000000000000001</v>
       </c>
-      <c r="AN17" s="12">
+      <c r="AN17" s="11">
         <v>1.2408299999999999E-5</v>
       </c>
       <c r="AO17">
@@ -7702,7 +7180,7 @@
       <c r="AM18">
         <v>1.47</v>
       </c>
-      <c r="AN18" s="12">
+      <c r="AN18" s="11">
         <v>4.0399199999999998E-5</v>
       </c>
       <c r="AO18">
@@ -7974,7 +7452,7 @@
       <c r="AM19">
         <v>1.36</v>
       </c>
-      <c r="AN19" s="12">
+      <c r="AN19" s="11">
         <v>2.7255060000000003E-4</v>
       </c>
       <c r="AO19">
@@ -8246,7 +7724,7 @@
       <c r="AM20">
         <v>1.19</v>
       </c>
-      <c r="AN20" s="12">
+      <c r="AN20" s="11">
         <v>2.6043090000000001E-4</v>
       </c>
       <c r="AO20">
@@ -8518,7 +7996,7 @@
       <c r="AM21">
         <v>1.48</v>
       </c>
-      <c r="AN21" s="12">
+      <c r="AN21" s="11">
         <v>5.3891999999999998E-5</v>
       </c>
       <c r="AO21">
@@ -8790,7 +8268,7 @@
       <c r="AM22">
         <v>1.27</v>
       </c>
-      <c r="AN22" s="12">
+      <c r="AN22" s="11">
         <v>6.237355E-4</v>
       </c>
       <c r="AO22">
@@ -9062,7 +8540,7 @@
       <c r="AM23">
         <v>1.25</v>
       </c>
-      <c r="AN23" s="12">
+      <c r="AN23" s="11">
         <v>3.0876600000000002E-5</v>
       </c>
       <c r="AO23">
@@ -9334,7 +8812,7 @@
       <c r="AM24">
         <v>1.22</v>
       </c>
-      <c r="AN24" s="12">
+      <c r="AN24" s="11">
         <v>3.622225E-4</v>
       </c>
       <c r="AO24">
@@ -9606,7 +9084,7 @@
       <c r="AM25">
         <v>1.66</v>
       </c>
-      <c r="AN25" s="12">
+      <c r="AN25" s="11">
         <v>8.80442E-5</v>
       </c>
       <c r="AO25">
@@ -9878,7 +9356,7 @@
       <c r="AM26">
         <v>1.38</v>
       </c>
-      <c r="AN26" s="12">
+      <c r="AN26" s="11">
         <v>9.2211000000000005E-6</v>
       </c>
       <c r="AO26">
@@ -10150,7 +9628,7 @@
       <c r="AM27">
         <v>1.08</v>
       </c>
-      <c r="AN27" s="12">
+      <c r="AN27" s="11">
         <v>1.1109071E-3</v>
       </c>
       <c r="AO27">
@@ -10422,7 +9900,7 @@
       <c r="AM28">
         <v>1.23</v>
       </c>
-      <c r="AN28" s="12">
+      <c r="AN28" s="11">
         <v>4.633649E-4</v>
       </c>
       <c r="AO28">
@@ -10694,7 +10172,7 @@
       <c r="AM29">
         <v>1.43</v>
       </c>
-      <c r="AN29" s="12">
+      <c r="AN29" s="11">
         <v>3.7294099999999999E-5</v>
       </c>
       <c r="AO29">
@@ -10966,7 +10444,7 @@
       <c r="AM30">
         <v>0.95</v>
       </c>
-      <c r="AN30" s="12">
+      <c r="AN30" s="11">
         <v>1.1065300000000001E-5</v>
       </c>
       <c r="AO30">
@@ -11238,7 +10716,7 @@
       <c r="AM31">
         <v>1.1000000000000001</v>
       </c>
-      <c r="AN31" s="12">
+      <c r="AN31" s="11">
         <v>1.87154E-5</v>
       </c>
       <c r="AO31">
@@ -11510,7 +10988,7 @@
       <c r="AM32">
         <v>1.67</v>
       </c>
-      <c r="AN32" s="12">
+      <c r="AN32" s="11">
         <v>1.094387E-4</v>
       </c>
       <c r="AO32">
@@ -11782,7 +11260,7 @@
       <c r="AM33">
         <v>1.5</v>
       </c>
-      <c r="AN33" s="12">
+      <c r="AN33" s="11">
         <v>7.7097630000000003E-4</v>
       </c>
       <c r="AO33">
@@ -12054,7 +11532,7 @@
       <c r="AM34">
         <v>1.38</v>
       </c>
-      <c r="AN34" s="12">
+      <c r="AN34" s="11">
         <v>8.5380000000000002E-6</v>
       </c>
       <c r="AO34">
@@ -12326,7 +11804,7 @@
       <c r="AM35">
         <v>1.27</v>
       </c>
-      <c r="AN35" s="12">
+      <c r="AN35" s="11">
         <v>2.5305799000000001E-3</v>
       </c>
       <c r="AO35">
@@ -12598,7 +12076,7 @@
       <c r="AM36">
         <v>1.42</v>
       </c>
-      <c r="AN36" s="12">
+      <c r="AN36" s="11">
         <v>2.1857399999999998E-5</v>
       </c>
       <c r="AO36">
@@ -12870,7 +12348,7 @@
       <c r="AM37">
         <v>0.92</v>
       </c>
-      <c r="AN37" s="12">
+      <c r="AN37" s="11">
         <v>4.227492E-4</v>
       </c>
       <c r="AO37">
@@ -13142,7 +12620,7 @@
       <c r="AM38">
         <v>1.1399999999999999</v>
       </c>
-      <c r="AN38" s="12">
+      <c r="AN38" s="11">
         <v>5.2309809999999998E-4</v>
       </c>
       <c r="AO38">
@@ -13414,7 +12892,7 @@
       <c r="AM39">
         <v>1.1000000000000001</v>
       </c>
-      <c r="AN39" s="12">
+      <c r="AN39" s="11">
         <v>2.0321542000000001E-3</v>
       </c>
       <c r="AO39">
@@ -13686,7 +13164,7 @@
       <c r="AM40">
         <v>1.23</v>
       </c>
-      <c r="AN40" s="12">
+      <c r="AN40" s="11">
         <v>1.1543419999999999E-4</v>
       </c>
       <c r="AO40">
@@ -13958,7 +13436,7 @@
       <c r="AM41">
         <v>1.35</v>
       </c>
-      <c r="AN41" s="12">
+      <c r="AN41" s="11">
         <v>5.0408499999999997E-5</v>
       </c>
       <c r="AO41">
@@ -14230,7 +13708,7 @@
       <c r="AM42">
         <v>1.42</v>
       </c>
-      <c r="AN42" s="12">
+      <c r="AN42" s="11">
         <v>6.5571999999999997E-6</v>
       </c>
       <c r="AO42">
@@ -14502,7 +13980,7 @@
       <c r="AM43">
         <v>1.1000000000000001</v>
       </c>
-      <c r="AN43" s="12">
+      <c r="AN43" s="11">
         <v>6.6186799999999995E-5</v>
       </c>
       <c r="AO43">
@@ -14774,7 +14252,7 @@
       <c r="AM44">
         <v>1.1399999999999999</v>
       </c>
-      <c r="AN44" s="12">
+      <c r="AN44" s="11">
         <v>1.382953E-4</v>
       </c>
       <c r="AO44">
@@ -15046,7 +14524,7 @@
       <c r="AM45">
         <v>1.17</v>
       </c>
-      <c r="AN45" s="12">
+      <c r="AN45" s="11">
         <v>2.0489999999999999E-7</v>
       </c>
       <c r="AO45">
@@ -15318,7 +14796,7 @@
       <c r="AM46">
         <v>1.27</v>
       </c>
-      <c r="AN46" s="12">
+      <c r="AN46" s="11">
         <v>1.5308429999999999E-4</v>
       </c>
       <c r="AO46">
@@ -15590,7 +15068,7 @@
       <c r="AM47">
         <v>1.0900000000000001</v>
       </c>
-      <c r="AN47" s="12">
+      <c r="AN47" s="11">
         <v>1.0042100000000001E-4</v>
       </c>
       <c r="AO47">
@@ -15862,7 +15340,7 @@
       <c r="AM48">
         <v>1.23</v>
       </c>
-      <c r="AN48" s="12">
+      <c r="AN48" s="11">
         <v>1.6604759999999999E-4</v>
       </c>
       <c r="AO48">
@@ -16134,7 +15612,7 @@
       <c r="AM49">
         <v>1.05</v>
       </c>
-      <c r="AN49" s="12">
+      <c r="AN49" s="11">
         <v>2.9587398E-3</v>
       </c>
       <c r="AO49">
@@ -16406,7 +15884,7 @@
       <c r="AM50">
         <v>1.21</v>
       </c>
-      <c r="AN50" s="12">
+      <c r="AN50" s="11">
         <v>7.0831499999999994E-5</v>
       </c>
       <c r="AO50">
@@ -16678,7 +16156,7 @@
       <c r="AM51">
         <v>1.5</v>
       </c>
-      <c r="AN51" s="12">
+      <c r="AN51" s="11">
         <v>1.949985E-4</v>
       </c>
       <c r="AO51">
@@ -16950,7 +16428,7 @@
       <c r="AM52">
         <v>1.45</v>
       </c>
-      <c r="AN52" s="12">
+      <c r="AN52" s="11">
         <v>2.5105200000000001E-5</v>
       </c>
       <c r="AO52">
@@ -17222,7 +16700,7 @@
       <c r="AM53">
         <v>1.39</v>
       </c>
-      <c r="AN53" s="12">
+      <c r="AN53" s="11">
         <v>1.217027E-4</v>
       </c>
       <c r="AO53">
@@ -17494,7 +16972,7 @@
       <c r="AM54">
         <v>1.77</v>
       </c>
-      <c r="AN54" s="12">
+      <c r="AN54" s="11">
         <v>7.4918960000000003E-4</v>
       </c>
       <c r="AO54">
@@ -17766,7 +17244,7 @@
       <c r="AM55">
         <v>1.26</v>
       </c>
-      <c r="AN55" s="12">
+      <c r="AN55" s="11">
         <v>5.4437979999999995E-4</v>
       </c>
       <c r="AO55">
@@ -18038,7 +17516,7 @@
       <c r="AM56">
         <v>1.51</v>
       </c>
-      <c r="AN56" s="12">
+      <c r="AN56" s="11">
         <v>2.5393800000000001E-5</v>
       </c>
       <c r="AO56">
@@ -18310,7 +17788,7 @@
       <c r="AM57">
         <v>1.39</v>
       </c>
-      <c r="AN57" s="12">
+      <c r="AN57" s="11">
         <v>4.5982999999999999E-4</v>
       </c>
       <c r="AO57">
@@ -18582,7 +18060,7 @@
       <c r="AM58">
         <v>1.28</v>
       </c>
-      <c r="AN58" s="12">
+      <c r="AN58" s="11">
         <v>2.9967006399999999E-2</v>
       </c>
       <c r="AO58">
@@ -18854,7 +18332,7 @@
       <c r="AM59">
         <v>1.1399999999999999</v>
       </c>
-      <c r="AN59" s="12">
+      <c r="AN59" s="11">
         <v>2.0363384000000001E-3</v>
       </c>
       <c r="AO59">
@@ -19126,7 +18604,7 @@
       <c r="AM60">
         <v>1.39</v>
       </c>
-      <c r="AN60" s="12">
+      <c r="AN60" s="11">
         <v>2.8869106000000001E-3</v>
       </c>
       <c r="AO60">
@@ -19398,7 +18876,7 @@
       <c r="AM61">
         <v>1.33</v>
       </c>
-      <c r="AN61" s="12">
+      <c r="AN61" s="11">
         <v>1.0809684E-3</v>
       </c>
       <c r="AO61">
@@ -19670,7 +19148,7 @@
       <c r="AM62">
         <v>1.17</v>
       </c>
-      <c r="AN62" s="12">
+      <c r="AN62" s="11">
         <v>3.3140368000000001E-3</v>
       </c>
       <c r="AO62">
@@ -19942,7 +19420,7 @@
       <c r="AM63">
         <v>1.72</v>
       </c>
-      <c r="AN63" s="12">
+      <c r="AN63" s="11">
         <v>2.7225484000000001E-3</v>
       </c>
       <c r="AO63">
@@ -20214,7 +19692,7 @@
       <c r="AM64">
         <v>0.99</v>
       </c>
-      <c r="AN64" s="12">
+      <c r="AN64" s="11">
         <v>9.7347760000000003E-4</v>
       </c>
       <c r="AO64">
@@ -20486,7 +19964,7 @@
       <c r="AM65">
         <v>1.71</v>
       </c>
-      <c r="AN65" s="12">
+      <c r="AN65" s="11">
         <v>3.6503600000000001E-5</v>
       </c>
       <c r="AO65">
@@ -20758,7 +20236,7 @@
       <c r="AM66">
         <v>1.63</v>
       </c>
-      <c r="AN66" s="12">
+      <c r="AN66" s="11">
         <v>6.1437152999999998E-3</v>
       </c>
       <c r="AO66">
@@ -21030,7 +20508,7 @@
       <c r="AM67">
         <v>1.7</v>
       </c>
-      <c r="AN67" s="12">
+      <c r="AN67" s="11">
         <v>1.8966E-4</v>
       </c>
       <c r="AO67">
@@ -21302,7 +20780,7 @@
       <c r="AM68">
         <v>1.54</v>
       </c>
-      <c r="AN68" s="12">
+      <c r="AN68" s="11">
         <v>2.5762454000000001E-3</v>
       </c>
       <c r="AO68">
@@ -21574,7 +21052,7 @@
       <c r="AM69">
         <v>1.31</v>
       </c>
-      <c r="AN69" s="12">
+      <c r="AN69" s="11">
         <v>1.0364571E-3</v>
       </c>
       <c r="AO69">
@@ -21846,7 +21324,7 @@
       <c r="AM70">
         <v>1.1200000000000001</v>
       </c>
-      <c r="AN70" s="12">
+      <c r="AN70" s="11">
         <v>2.9621299999999998E-4</v>
       </c>
       <c r="AO70">
@@ -22118,7 +21596,7 @@
       <c r="AM71">
         <v>1.28</v>
       </c>
-      <c r="AN71" s="12">
+      <c r="AN71" s="11">
         <v>4.511009E-4</v>
       </c>
       <c r="AO71">
@@ -22390,7 +21868,7 @@
       <c r="AM72">
         <v>1.52</v>
       </c>
-      <c r="AN72" s="12">
+      <c r="AN72" s="11">
         <v>1.8665894E-3</v>
       </c>
       <c r="AO72">
@@ -22662,7 +22140,7 @@
       <c r="AM73">
         <v>1.58</v>
       </c>
-      <c r="AN73" s="12">
+      <c r="AN73" s="11">
         <v>3.1889434000000002E-3</v>
       </c>
       <c r="AO73">
@@ -22934,7 +22412,7 @@
       <c r="AM74">
         <v>1.54</v>
       </c>
-      <c r="AN74" s="12">
+      <c r="AN74" s="11">
         <v>2.9549159999999998E-4</v>
       </c>
       <c r="AO74">
@@ -23206,7 +22684,7 @@
       <c r="AM75">
         <v>1.53</v>
       </c>
-      <c r="AN75" s="12">
+      <c r="AN75" s="11">
         <v>1.41251629E-2</v>
       </c>
       <c r="AO75">
@@ -23478,7 +22956,7 @@
       <c r="AM76">
         <v>1.38</v>
       </c>
-      <c r="AN76" s="12">
+      <c r="AN76" s="11">
         <v>4.2130599999999999E-5</v>
       </c>
       <c r="AO76">
@@ -23750,7 +23228,7 @@
       <c r="AM77">
         <v>1.1499999999999999</v>
       </c>
-      <c r="AN77" s="12">
+      <c r="AN77" s="11">
         <v>8.6425499999999994E-5</v>
       </c>
       <c r="AO77">
@@ -24022,7 +23500,7 @@
       <c r="AM78">
         <v>1.28</v>
       </c>
-      <c r="AN78" s="12">
+      <c r="AN78" s="11">
         <v>4.8637810000000002E-4</v>
       </c>
       <c r="AO78">
@@ -24294,7 +23772,7 @@
       <c r="AM79">
         <v>1.33</v>
       </c>
-      <c r="AN79" s="12">
+      <c r="AN79" s="11">
         <v>3.74501E-3</v>
       </c>
       <c r="AO79">
@@ -24566,7 +24044,7 @@
       <c r="AM80">
         <v>1.1000000000000001</v>
       </c>
-      <c r="AN80" s="12">
+      <c r="AN80" s="11">
         <v>3.9925380000000002E-4</v>
       </c>
       <c r="AO80">
@@ -24838,7 +24316,7 @@
       <c r="AM81">
         <v>1.24</v>
       </c>
-      <c r="AN81" s="12">
+      <c r="AN81" s="11">
         <v>2.1617924999999998E-3</v>
       </c>
       <c r="AO81">
@@ -25110,7 +24588,7 @@
       <c r="AM82">
         <v>1.18</v>
       </c>
-      <c r="AN82" s="12">
+      <c r="AN82" s="11">
         <v>3.724666E-4</v>
       </c>
       <c r="AO82">
@@ -25382,7 +24860,7 @@
       <c r="AM83">
         <v>1.41</v>
       </c>
-      <c r="AN83" s="12">
+      <c r="AN83" s="11">
         <v>8.3467730000000003E-4</v>
       </c>
       <c r="AO83">
@@ -25654,7 +25132,7 @@
       <c r="AM84">
         <v>1.43</v>
       </c>
-      <c r="AN84" s="12">
+      <c r="AN84" s="11">
         <v>3.728995E-4</v>
       </c>
       <c r="AO84">
@@ -25926,7 +25404,7 @@
       <c r="AM85">
         <v>1.34</v>
       </c>
-      <c r="AN85" s="12">
+      <c r="AN85" s="11">
         <v>2.9431572000000001E-3</v>
       </c>
       <c r="AO85">
@@ -26198,7 +25676,7 @@
       <c r="AM86">
         <v>1.58</v>
       </c>
-      <c r="AN86" s="12">
+      <c r="AN86" s="11">
         <v>1.21155892E-2</v>
       </c>
       <c r="AO86">
@@ -26470,7 +25948,7 @@
       <c r="AM87">
         <v>1.6</v>
       </c>
-      <c r="AN87" s="12">
+      <c r="AN87" s="11">
         <v>4.5492429999999999E-4</v>
       </c>
       <c r="AO87">
@@ -26742,7 +26220,7 @@
       <c r="AM88">
         <v>1.43</v>
       </c>
-      <c r="AN88" s="12">
+      <c r="AN88" s="11">
         <v>7.5568230000000003E-4</v>
       </c>
       <c r="AO88">
@@ -27014,7 +26492,7 @@
       <c r="AM89">
         <v>1.39</v>
       </c>
-      <c r="AN89" s="12">
+      <c r="AN89" s="11">
         <v>1.1024666000000001E-3</v>
       </c>
       <c r="AO89">
@@ -27286,7 +26764,7 @@
       <c r="AM90">
         <v>1.35</v>
       </c>
-      <c r="AN90" s="12">
+      <c r="AN90" s="11">
         <v>8.1079839999999997E-4</v>
       </c>
       <c r="AO90">
@@ -27558,7 +27036,7 @@
       <c r="AM91">
         <v>1.79</v>
       </c>
-      <c r="AN91" s="12">
+      <c r="AN91" s="11">
         <v>1.235063E-4</v>
       </c>
       <c r="AO91">
@@ -27830,7 +27308,7 @@
       <c r="AM92">
         <v>1.43</v>
       </c>
-      <c r="AN92" s="12">
+      <c r="AN92" s="11">
         <v>3.0018079999999999E-4</v>
       </c>
       <c r="AO92">
@@ -28102,7 +27580,7 @@
       <c r="AM93">
         <v>1.43</v>
       </c>
-      <c r="AN93" s="12">
+      <c r="AN93" s="11">
         <v>2.5155022999999999E-3</v>
       </c>
       <c r="AO93">
@@ -28374,7 +27852,7 @@
       <c r="AM94">
         <v>1.23</v>
       </c>
-      <c r="AN94" s="12">
+      <c r="AN94" s="11">
         <v>1.46854E-5</v>
       </c>
       <c r="AO94">
@@ -28646,7 +28124,7 @@
       <c r="AM95">
         <v>1.53</v>
       </c>
-      <c r="AN95" s="12">
+      <c r="AN95" s="11">
         <v>3.2158521E-3</v>
       </c>
       <c r="AO95">
@@ -28918,7 +28396,7 @@
       <c r="AM96">
         <v>1.27</v>
       </c>
-      <c r="AN96" s="12">
+      <c r="AN96" s="11">
         <v>3.6331909E-3</v>
       </c>
       <c r="AO96">
@@ -29190,7 +28668,7 @@
       <c r="AM97">
         <v>1.44</v>
       </c>
-      <c r="AN97" s="12">
+      <c r="AN97" s="11">
         <v>3.9718951000000001E-3</v>
       </c>
       <c r="AO97">
@@ -29462,7 +28940,7 @@
       <c r="AM98">
         <v>1.58</v>
       </c>
-      <c r="AN98" s="12">
+      <c r="AN98" s="11">
         <v>2.54736718E-2</v>
       </c>
       <c r="AO98">
@@ -29734,7 +29212,7 @@
       <c r="AM99">
         <v>1.68</v>
       </c>
-      <c r="AN99" s="12">
+      <c r="AN99" s="11">
         <v>8.7250824000000005E-3</v>
       </c>
       <c r="AO99">
@@ -30006,7 +29484,7 @@
       <c r="AM100">
         <v>1.36</v>
       </c>
-      <c r="AN100" s="12">
+      <c r="AN100" s="11">
         <v>3.7784117E-3</v>
       </c>
       <c r="AO100">
@@ -30278,7 +29756,7 @@
       <c r="AM101">
         <v>1.2</v>
       </c>
-      <c r="AN101" s="12">
+      <c r="AN101" s="11">
         <v>4.5672790000000002E-4</v>
       </c>
       <c r="AO101">
@@ -30550,7 +30028,7 @@
       <c r="AM102">
         <v>1.39</v>
       </c>
-      <c r="AN102" s="12">
+      <c r="AN102" s="11">
         <v>1.99561444E-2</v>
       </c>
       <c r="AO102">
@@ -30822,7 +30300,7 @@
       <c r="AM103">
         <v>1.34</v>
       </c>
-      <c r="AN103" s="12">
+      <c r="AN103" s="11">
         <v>1.0024063000000001E-3</v>
       </c>
       <c r="AO103">
@@ -31094,7 +30572,7 @@
       <c r="AM104">
         <v>1.39</v>
       </c>
-      <c r="AN104" s="12">
+      <c r="AN104" s="11">
         <v>3.7963025999999999E-3</v>
       </c>
       <c r="AO104">
@@ -31366,7 +30844,7 @@
       <c r="AM105">
         <v>1.21</v>
       </c>
-      <c r="AN105" s="12">
+      <c r="AN105" s="11">
         <v>5.61982E-5</v>
       </c>
       <c r="AO105">
@@ -31638,7 +31116,7 @@
       <c r="AM106">
         <v>1.36</v>
       </c>
-      <c r="AN106" s="12">
+      <c r="AN106" s="11">
         <v>9.9411000000000001E-5</v>
       </c>
       <c r="AO106">
@@ -31910,7 +31388,7 @@
       <c r="AM107">
         <v>1.37</v>
       </c>
-      <c r="AN107" s="12">
+      <c r="AN107" s="11">
         <v>1.9815060000000001E-4</v>
       </c>
       <c r="AO107">
@@ -32182,7 +31660,7 @@
       <c r="AM108">
         <v>1.4</v>
       </c>
-      <c r="AN108" s="12">
+      <c r="AN108" s="11">
         <v>1.5488780000000001E-4</v>
       </c>
       <c r="AO108">
@@ -32454,7 +31932,7 @@
       <c r="AM109">
         <v>1.1000000000000001</v>
       </c>
-      <c r="AN109" s="12">
+      <c r="AN109" s="11">
         <v>1.7238502900000001E-2</v>
       </c>
       <c r="AO109">
@@ -32726,7 +32204,7 @@
       <c r="AM110">
         <v>1.45</v>
       </c>
-      <c r="AN110" s="12">
+      <c r="AN110" s="11">
         <v>1.9944962000000002E-3</v>
       </c>
       <c r="AO110">
@@ -32998,7 +32476,7 @@
       <c r="AM111">
         <v>1.54</v>
       </c>
-      <c r="AN111" s="13">
+      <c r="AN111" s="12">
         <v>3.0588000000000002E-4</v>
       </c>
       <c r="AO111">
@@ -33270,7 +32748,7 @@
       <c r="AM112">
         <v>1.71</v>
       </c>
-      <c r="AN112" s="12">
+      <c r="AN112" s="11">
         <v>4.6098399999999999E-5</v>
       </c>
       <c r="AO112">
@@ -33542,7 +33020,7 @@
       <c r="AM113">
         <v>1.67</v>
       </c>
-      <c r="AN113" s="12">
+      <c r="AN113" s="11">
         <v>1.4536510000000001E-4</v>
       </c>
       <c r="AO113">
@@ -33814,7 +33292,7 @@
       <c r="AM114">
         <v>1.57</v>
       </c>
-      <c r="AN114" s="12">
+      <c r="AN114" s="11">
         <v>4.4936949999999998E-4</v>
       </c>
       <c r="AO114">
@@ -34086,7 +33564,7 @@
       <c r="AM115">
         <v>1.76</v>
       </c>
-      <c r="AN115" s="12">
+      <c r="AN115" s="11">
         <v>2.0920999999999998E-5</v>
       </c>
       <c r="AO115">
@@ -34358,7 +33836,7 @@
       <c r="AM116">
         <v>1.52</v>
       </c>
-      <c r="AN116" s="13">
+      <c r="AN116" s="12">
         <v>1.563306E-4</v>
       </c>
       <c r="AO116">
@@ -34630,7 +34108,7 @@
       <c r="AM117">
         <v>1.43</v>
       </c>
-      <c r="AN117" s="12">
+      <c r="AN117" s="11">
         <v>2.2808259000000001E-3</v>
       </c>
       <c r="AO117">
@@ -34902,7 +34380,7 @@
       <c r="AM118">
         <v>1.57</v>
       </c>
-      <c r="AN118" s="12">
+      <c r="AN118" s="11">
         <v>3.5443120000000001E-4</v>
       </c>
       <c r="AO118">
@@ -35174,7 +34652,7 @@
       <c r="AM119">
         <v>1.85</v>
       </c>
-      <c r="AN119" s="12">
+      <c r="AN119" s="11">
         <v>5.7612210000000002E-4</v>
       </c>
       <c r="AO119">
@@ -35446,7 +34924,7 @@
       <c r="AM120">
         <v>1.31</v>
       </c>
-      <c r="AN120" s="12">
+      <c r="AN120" s="11">
         <v>5.8218199999999998E-5</v>
       </c>
       <c r="AO120">
@@ -35718,7 +35196,7 @@
       <c r="AM121">
         <v>1.54</v>
       </c>
-      <c r="AN121" s="12">
+      <c r="AN121" s="11">
         <v>2.0134696000000001E-3</v>
       </c>
       <c r="AO121">
@@ -35990,7 +35468,7 @@
       <c r="AM122">
         <v>1.48</v>
       </c>
-      <c r="AN122" s="12">
+      <c r="AN122" s="11">
         <v>7.9305160000000001E-4</v>
       </c>
       <c r="AO122">
@@ -36262,7 +35740,7 @@
       <c r="AM123">
         <v>1.43</v>
       </c>
-      <c r="AN123" s="12">
+      <c r="AN123" s="11">
         <v>2.3143E-4</v>
       </c>
       <c r="AO123">
@@ -36534,7 +36012,7 @@
       <c r="AM124">
         <v>1.5</v>
       </c>
-      <c r="AN124" s="12">
+      <c r="AN124" s="11">
         <v>1.3060787799999999E-2</v>
       </c>
       <c r="AO124">
@@ -36806,7 +36284,7 @@
       <c r="AM125">
         <v>1.47</v>
       </c>
-      <c r="AN125" s="12">
+      <c r="AN125" s="11">
         <v>4.298913E-4</v>
       </c>
       <c r="AO125">
@@ -37078,7 +36556,7 @@
       <c r="AM126">
         <v>1.57</v>
       </c>
-      <c r="AN126" s="12">
+      <c r="AN126" s="11">
         <v>2.9008823000000001E-3</v>
       </c>
       <c r="AO126">
@@ -37350,7 +36828,7 @@
       <c r="AM127">
         <v>1.43</v>
       </c>
-      <c r="AN127" s="12">
+      <c r="AN127" s="11">
         <v>3.9894300000000002E-5</v>
       </c>
       <c r="AO127">
@@ -37622,7 +37100,7 @@
       <c r="AM128">
         <v>1.79</v>
       </c>
-      <c r="AN128" s="12">
+      <c r="AN128" s="11">
         <v>1.8201299999999999E-4</v>
       </c>
       <c r="AO128">
@@ -37894,7 +37372,7 @@
       <c r="AM129">
         <v>1.29</v>
       </c>
-      <c r="AN129" s="12">
+      <c r="AN129" s="11">
         <v>1.5914419999999999E-4</v>
       </c>
       <c r="AO129">
@@ -38166,7 +37644,7 @@
       <c r="AM130">
         <v>1.21</v>
       </c>
-      <c r="AN130" s="12">
+      <c r="AN130" s="11">
         <v>1.2553344E-3</v>
       </c>
       <c r="AO130">
@@ -38438,7 +37916,7 @@
       <c r="AM131">
         <v>1.59</v>
       </c>
-      <c r="AN131" s="12">
+      <c r="AN131" s="11">
         <v>3.1814399999999998E-5</v>
       </c>
       <c r="AO131">
@@ -38710,7 +38188,7 @@
       <c r="AM132">
         <v>1.25</v>
       </c>
-      <c r="AN132" s="12">
+      <c r="AN132" s="11">
         <v>1.398824E-4</v>
       </c>
       <c r="AO132">
@@ -38982,7 +38460,7 @@
       <c r="AM133">
         <v>1.68</v>
       </c>
-      <c r="AN133" s="12">
+      <c r="AN133" s="11">
         <v>3.4346570000000001E-4</v>
       </c>
       <c r="AO133">
@@ -39254,7 +38732,7 @@
       <c r="AM134">
         <v>1.36</v>
       </c>
-      <c r="AN134" s="12">
+      <c r="AN134" s="11">
         <v>4.5809858000000004E-3</v>
       </c>
       <c r="AO134">
@@ -39526,7 +39004,7 @@
       <c r="AM135">
         <v>1.39</v>
       </c>
-      <c r="AN135" s="12">
+      <c r="AN135" s="11">
         <v>6.1753099999999997E-5</v>
       </c>
       <c r="AO135">
@@ -39798,7 +39276,7 @@
       <c r="AM136">
         <v>1.32</v>
       </c>
-      <c r="AN136" s="12">
+      <c r="AN136" s="11">
         <v>7.1600449999999996E-4</v>
       </c>
       <c r="AO136">
@@ -40070,7 +39548,7 @@
       <c r="AM137">
         <v>1.62</v>
       </c>
-      <c r="AN137" s="12">
+      <c r="AN137" s="11">
         <v>1.0894811E-3</v>
       </c>
       <c r="AO137">
@@ -40342,7 +39820,7 @@
       <c r="AM138">
         <v>1.54</v>
       </c>
-      <c r="AN138" s="12">
+      <c r="AN138" s="11">
         <v>4.5066799999999999E-4</v>
       </c>
       <c r="AO138">
@@ -40614,7 +40092,7 @@
       <c r="AM139">
         <v>1.31</v>
       </c>
-      <c r="AN139" s="12">
+      <c r="AN139" s="11">
         <v>4.7334207999999997E-3</v>
       </c>
       <c r="AO139">
@@ -40886,7 +40364,7 @@
       <c r="AM140">
         <v>1.53</v>
       </c>
-      <c r="AN140" s="12">
+      <c r="AN140" s="11">
         <v>7.4846820000000003E-4</v>
       </c>
       <c r="AO140">
@@ -41158,7 +40636,7 @@
       <c r="AM141">
         <v>1.37</v>
       </c>
-      <c r="AN141" s="12">
+      <c r="AN141" s="11">
         <v>2.6172940000000002E-4</v>
       </c>
       <c r="AO141">
@@ -41430,7 +40908,7 @@
       <c r="AM142">
         <v>1.64</v>
       </c>
-      <c r="AN142" s="12">
+      <c r="AN142" s="11">
         <v>1.3667209E-3</v>
       </c>
       <c r="AO142">
@@ -41702,7 +41180,7 @@
       <c r="AM143">
         <v>1.47</v>
       </c>
-      <c r="AN143" s="12">
+      <c r="AN143" s="11">
         <v>1.5862114399999998E-2</v>
       </c>
       <c r="AO143">
@@ -41974,7 +41452,7 @@
       <c r="AM144">
         <v>1.67</v>
       </c>
-      <c r="AN144" s="12">
+      <c r="AN144" s="11">
         <v>3.508963E-4</v>
       </c>
       <c r="AO144">
@@ -42246,7 +41724,7 @@
       <c r="AM145">
         <v>1.32</v>
       </c>
-      <c r="AN145" s="12">
+      <c r="AN145" s="11">
         <v>2.5222114E-3</v>
       </c>
       <c r="AO145">
@@ -42518,7 +41996,7 @@
       <c r="AM146">
         <v>1.31</v>
       </c>
-      <c r="AN146" s="12">
+      <c r="AN146" s="11">
         <v>2.4121877999999999E-2</v>
       </c>
       <c r="AO146">
@@ -42790,7 +42268,7 @@
       <c r="AM147">
         <v>1.39</v>
       </c>
-      <c r="AN147" s="12">
+      <c r="AN147" s="11">
         <v>7.8461109999999998E-4</v>
       </c>
       <c r="AO147">
@@ -43062,7 +42540,7 @@
       <c r="AM148">
         <v>1.63</v>
       </c>
-      <c r="AN148" s="12">
+      <c r="AN148" s="11">
         <v>2.0842402999999999E-3</v>
       </c>
       <c r="AO148">
@@ -43334,7 +42812,7 @@
       <c r="AM149">
         <v>1.7</v>
       </c>
-      <c r="AN149" s="12">
+      <c r="AN149" s="11">
         <v>1.1282929999999999E-4</v>
       </c>
       <c r="AO149">
@@ -43606,7 +43084,7 @@
       <c r="AM150">
         <v>1.52</v>
       </c>
-      <c r="AN150" s="12">
+      <c r="AN150" s="11">
         <v>1.4514869999999999E-4</v>
       </c>
       <c r="AO150">
@@ -43878,7 +43356,7 @@
       <c r="AM151">
         <v>1.59</v>
       </c>
-      <c r="AN151" s="12">
+      <c r="AN151" s="11">
         <v>8.9903471000000006E-3</v>
       </c>
       <c r="AO151">
@@ -44150,7 +43628,7 @@
       <c r="AM152">
         <v>1.36</v>
       </c>
-      <c r="AN152" s="12">
+      <c r="AN152" s="11">
         <v>4.7663890000000002E-4</v>
       </c>
       <c r="AO152">
@@ -44422,7 +43900,7 @@
       <c r="AM153">
         <v>1.56</v>
       </c>
-      <c r="AN153" s="12">
+      <c r="AN153" s="11">
         <v>2.26524E-5</v>
       </c>
       <c r="AO153">
@@ -44694,7 +44172,7 @@
       <c r="AM154">
         <v>1.29</v>
       </c>
-      <c r="AN154" s="12">
+      <c r="AN154" s="11">
         <v>5.8326410000000004E-4</v>
       </c>
       <c r="AO154">
@@ -44966,7 +44444,7 @@
       <c r="AM155">
         <v>1.07</v>
       </c>
-      <c r="AN155" s="12">
+      <c r="AN155" s="11">
         <v>7.7912799999999997E-5</v>
       </c>
       <c r="AO155">
@@ -45238,7 +44716,7 @@
       <c r="AM156">
         <v>1.56</v>
       </c>
-      <c r="AN156" s="12">
+      <c r="AN156" s="11">
         <v>6.5439559999999999E-4</v>
       </c>
       <c r="AO156">
@@ -45510,7 +44988,7 @@
       <c r="AM157">
         <v>1.1200000000000001</v>
       </c>
-      <c r="AN157" s="12">
+      <c r="AN157" s="11">
         <v>1.3346199999999999E-5</v>
       </c>
       <c r="AO157">
@@ -45782,7 +45260,7 @@
       <c r="AM158">
         <v>1.62</v>
       </c>
-      <c r="AN158" s="12">
+      <c r="AN158" s="11">
         <v>2.0509829999999999E-4</v>
       </c>
       <c r="AO158">
@@ -46054,7 +45532,7 @@
       <c r="AM159">
         <v>1.1200000000000001</v>
       </c>
-      <c r="AN159" s="12">
+      <c r="AN159" s="11">
         <v>5.1949099999999996E-4</v>
       </c>
       <c r="AO159">
@@ -46326,7 +45804,7 @@
       <c r="AM160">
         <v>0.88</v>
       </c>
-      <c r="AN160" s="12">
+      <c r="AN160" s="11">
         <v>5.4505795999999999E-3</v>
       </c>
       <c r="AO160">
@@ -46598,7 +46076,7 @@
       <c r="AM161">
         <v>1.53</v>
       </c>
-      <c r="AN161" s="12">
+      <c r="AN161" s="11">
         <v>3.6712810000000002E-4</v>
       </c>
       <c r="AO161">
@@ -46870,7 +46348,7 @@
       <c r="AM162">
         <v>1.24</v>
       </c>
-      <c r="AN162" s="12">
+      <c r="AN162" s="11">
         <v>4.0464893E-3</v>
       </c>
       <c r="AO162">
@@ -47142,7 +46620,7 @@
       <c r="AM163">
         <v>1.19</v>
       </c>
-      <c r="AN163" s="12">
+      <c r="AN163" s="11">
         <v>2.0123874000000002E-3</v>
       </c>
       <c r="AO163">
@@ -47414,7 +46892,7 @@
       <c r="AM164">
         <v>1.7</v>
       </c>
-      <c r="AN164" s="12">
+      <c r="AN164" s="11">
         <v>6.8238659999999998E-4</v>
       </c>
       <c r="AO164">
@@ -47686,7 +47164,7 @@
       <c r="AM165">
         <v>1.21</v>
       </c>
-      <c r="AN165" s="12">
+      <c r="AN165" s="11">
         <v>1.4507657E-2</v>
       </c>
       <c r="AO165">
@@ -47958,7 +47436,7 @@
       <c r="AM166">
         <v>1.33</v>
       </c>
-      <c r="AN166" s="12">
+      <c r="AN166" s="11">
         <v>7.9860599999999999E-5</v>
       </c>
       <c r="AO166">
@@ -48230,7 +47708,7 @@
       <c r="AM167">
         <v>1.31</v>
       </c>
-      <c r="AN167" s="12">
+      <c r="AN167" s="11">
         <v>1.6852260000000001E-4</v>
       </c>
       <c r="AO167">
@@ -48502,7 +47980,7 @@
       <c r="AM168">
         <v>1.28</v>
       </c>
-      <c r="AN168" s="12">
+      <c r="AN168" s="11">
         <v>2.0501895000000002E-3</v>
       </c>
       <c r="AO168">
@@ -48774,7 +48252,7 @@
       <c r="AM169">
         <v>1.37</v>
       </c>
-      <c r="AN169" s="12">
+      <c r="AN169" s="11">
         <v>5.207174E-4</v>
       </c>
       <c r="AO169">
@@ -49046,7 +48524,7 @@
       <c r="AM170">
         <v>1.3</v>
       </c>
-      <c r="AN170" s="12">
+      <c r="AN170" s="11">
         <v>1.135507E-4</v>
       </c>
       <c r="AO170">
@@ -49318,7 +48796,7 @@
       <c r="AM171">
         <v>1.22</v>
       </c>
-      <c r="AN171" s="12">
+      <c r="AN171" s="11">
         <v>1.9139140000000001E-4</v>
       </c>
       <c r="AO171">
@@ -49590,7 +49068,7 @@
       <c r="AM172">
         <v>1.28</v>
       </c>
-      <c r="AN172" s="12">
+      <c r="AN172" s="11">
         <v>1.1910559999999999E-4</v>
       </c>
       <c r="AO172">
@@ -49862,7 +49340,7 @@
       <c r="AM173">
         <v>1.31</v>
       </c>
-      <c r="AN173" s="12">
+      <c r="AN173" s="11">
         <v>3.3906509999999997E-4</v>
       </c>
       <c r="AO173">
@@ -50134,7 +49612,7 @@
       <c r="AM174">
         <v>0.91</v>
       </c>
-      <c r="AN174" s="12">
+      <c r="AN174" s="11">
         <v>3.2512799999999998E-5</v>
       </c>
       <c r="AO174">
@@ -50406,7 +49884,7 @@
       <c r="AM175">
         <v>1.57</v>
       </c>
-      <c r="AN175" s="12">
+      <c r="AN175" s="11">
         <v>1.214142E-4</v>
       </c>
       <c r="AO175">
@@ -50678,7 +50156,7 @@
       <c r="AM176">
         <v>1.2</v>
       </c>
-      <c r="AN176" s="12">
+      <c r="AN176" s="11">
         <v>2.5718449999999999E-4</v>
       </c>
       <c r="AO176">
@@ -50950,7 +50428,7 @@
       <c r="AM177">
         <v>1.41</v>
       </c>
-      <c r="AN177" s="12">
+      <c r="AN177" s="11">
         <v>1.587835E-4</v>
       </c>
       <c r="AO177">
@@ -51222,7 +50700,7 @@
       <c r="AM178">
         <v>1.1499999999999999</v>
       </c>
-      <c r="AN178" s="12">
+      <c r="AN178" s="11">
         <v>6.6348549999999996E-4</v>
       </c>
       <c r="AO178">
@@ -51494,7 +50972,7 @@
       <c r="AM179">
         <v>1.47</v>
       </c>
-      <c r="AN179" s="12">
+      <c r="AN179" s="11">
         <v>6.462436E-4</v>
       </c>
       <c r="AO179">
@@ -51766,7 +51244,7 @@
       <c r="AM180">
         <v>0.81</v>
       </c>
-      <c r="AN180" s="12">
+      <c r="AN180" s="11">
         <v>1.5443333E-3</v>
       </c>
       <c r="AO180">
@@ -52038,7 +51516,7 @@
       <c r="AM181">
         <v>1.57</v>
       </c>
-      <c r="AN181" s="12">
+      <c r="AN181" s="11">
         <v>6.9075500000000004E-4</v>
       </c>
       <c r="AO181">
@@ -52310,7 +51788,7 @@
       <c r="AM182">
         <v>1</v>
       </c>
-      <c r="AN182" s="12">
+      <c r="AN182" s="11">
         <v>6.7740879999999995E-4</v>
       </c>
       <c r="AO182">
@@ -52582,7 +52060,7 @@
       <c r="AM183">
         <v>1.28</v>
       </c>
-      <c r="AN183" s="12">
+      <c r="AN183" s="11">
         <v>2.7002569999999999E-4</v>
       </c>
       <c r="AO183">
@@ -52854,7 +52332,7 @@
       <c r="AM184">
         <v>1.1200000000000001</v>
       </c>
-      <c r="AN184" s="12">
+      <c r="AN184" s="11">
         <v>1.05327E-5</v>
       </c>
       <c r="AO184">
@@ -53126,7 +52604,7 @@
       <c r="AM185">
         <v>1.1499999999999999</v>
       </c>
-      <c r="AN185" s="12">
+      <c r="AN185" s="11">
         <v>8.7224499999999998E-5</v>
       </c>
       <c r="AO185">
@@ -53398,7 +52876,7 @@
       <c r="AM186">
         <v>1.21</v>
       </c>
-      <c r="AN186" s="12">
+      <c r="AN186" s="11">
         <v>3.6777739999999999E-4</v>
       </c>
       <c r="AO186">
@@ -53670,7 +53148,7 @@
       <c r="AM187">
         <v>1.57</v>
       </c>
-      <c r="AN187" s="12">
+      <c r="AN187" s="11">
         <v>4.94891E-5</v>
       </c>
       <c r="AO187">
@@ -53942,7 +53420,7 @@
       <c r="AM188">
         <v>1.25</v>
       </c>
-      <c r="AN188" s="12">
+      <c r="AN188" s="11">
         <v>1.527236E-4</v>
       </c>
       <c r="AO188">
@@ -54214,7 +53692,7 @@
       <c r="AM189">
         <v>1.34</v>
       </c>
-      <c r="AN189" s="12">
+      <c r="AN189" s="11">
         <v>1.5380569999999999E-4</v>
       </c>
       <c r="AO189">
@@ -54486,7 +53964,7 @@
       <c r="AM190">
         <v>1.46</v>
       </c>
-      <c r="AN190" s="12">
+      <c r="AN190" s="11">
         <v>1.2903230999999999E-3</v>
       </c>
       <c r="AO190">
@@ -54758,7 +54236,7 @@
       <c r="AM191">
         <v>1.32</v>
       </c>
-      <c r="AN191" s="12">
+      <c r="AN191" s="11">
         <v>4.4655589999999999E-4</v>
       </c>
       <c r="AO191">
@@ -55030,7 +54508,7 @@
       <c r="AM192">
         <v>1.27</v>
       </c>
-      <c r="AN192" s="12">
+      <c r="AN192" s="11">
         <v>2.361191E-4</v>
       </c>
       <c r="AO192">
@@ -55302,7 +54780,7 @@
       <c r="AM193">
         <v>1.5</v>
       </c>
-      <c r="AN193" s="12">
+      <c r="AN193" s="11">
         <v>6.4573859999999996E-4</v>
       </c>
       <c r="AO193">
@@ -55574,7 +55052,7 @@
       <c r="AM194">
         <v>1.5</v>
       </c>
-      <c r="AN194" s="12">
+      <c r="AN194" s="11">
         <v>9.3957824000000002E-3</v>
       </c>
       <c r="AO194">
@@ -55846,7 +55324,7 @@
       <c r="AM195">
         <v>1.53</v>
       </c>
-      <c r="AN195" s="12">
+      <c r="AN195" s="11">
         <v>4.8883080000000005E-4</v>
       </c>
       <c r="AO195">
@@ -56118,7 +55596,7 @@
       <c r="AM196">
         <v>1.33</v>
       </c>
-      <c r="AN196" s="12">
+      <c r="AN196" s="11">
         <v>3.9677800000000002E-5</v>
       </c>
       <c r="AO196">
@@ -56390,7 +55868,7 @@
       <c r="AM197">
         <v>1.21</v>
       </c>
-      <c r="AN197" s="12">
+      <c r="AN197" s="11">
         <v>8.617303E-4</v>
       </c>
       <c r="AO197">
@@ -56662,7 +56140,7 @@
       <c r="AM198">
         <v>1.46</v>
       </c>
-      <c r="AN198" s="12">
+      <c r="AN198" s="11">
         <v>2.7877644E-3</v>
       </c>
       <c r="AO198">
@@ -56934,7 +56412,7 @@
       <c r="AM199">
         <v>1.07</v>
       </c>
-      <c r="AN199" s="12">
+      <c r="AN199" s="11">
         <v>2.2073857999999999E-3</v>
       </c>
       <c r="AO199">
@@ -57206,7 +56684,7 @@
       <c r="AM200">
         <v>1.18</v>
       </c>
-      <c r="AN200" s="12">
+      <c r="AN200" s="11">
         <v>5.0426900000000003E-5</v>
       </c>
       <c r="AO200">
@@ -57478,7 +56956,7 @@
       <c r="AM201">
         <v>1.22</v>
       </c>
-      <c r="AN201" s="12">
+      <c r="AN201" s="11">
         <v>1.07491E-5</v>
       </c>
       <c r="AO201">
@@ -57640,4 +57118,796 @@
   <phoneticPr fontId="5" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1E213513-60BC-A545-BBC0-EED3A764549D}">
+  <dimension ref="A1:D105"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="14" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="18.5" style="10" customWidth="1"/>
+    <col min="2" max="2" width="137.33203125" style="2" bestFit="1" customWidth="1"/>
+    <col min="3" max="16384" width="8.6640625" style="2"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A1" s="14" t="s">
+        <v>451</v>
+      </c>
+      <c r="B1" s="14"/>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A3" s="3"/>
+      <c r="B3" s="4"/>
+    </row>
+    <row r="4" spans="1:2" ht="15" x14ac:dyDescent="0.2">
+      <c r="A4" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="B4" s="5" t="s">
+        <v>543</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" ht="15" x14ac:dyDescent="0.2">
+      <c r="A5" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="B5" s="4" t="s">
+        <v>452</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" ht="15" x14ac:dyDescent="0.2">
+      <c r="A6" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="B6" s="4" t="s">
+        <v>453</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" ht="15" x14ac:dyDescent="0.2">
+      <c r="A7" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="B7" s="4" t="s">
+        <v>454</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" ht="15" x14ac:dyDescent="0.2">
+      <c r="A8" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="B8" s="4" t="s">
+        <v>455</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" ht="15" x14ac:dyDescent="0.2">
+      <c r="A9" s="6" t="s">
+        <v>5</v>
+      </c>
+      <c r="B9" s="4" t="s">
+        <v>456</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" ht="15" x14ac:dyDescent="0.2">
+      <c r="A10" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="B10" s="4" t="s">
+        <v>457</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" ht="15" x14ac:dyDescent="0.2">
+      <c r="A11" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="B11" s="4" t="s">
+        <v>458</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" ht="15" x14ac:dyDescent="0.2">
+      <c r="A12" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="B12" s="4" t="s">
+        <v>459</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2" ht="15" x14ac:dyDescent="0.2">
+      <c r="A13" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="B13" s="4" t="s">
+        <v>460</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2" ht="15" x14ac:dyDescent="0.2">
+      <c r="A14" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="B14" s="4" t="s">
+        <v>461</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2" ht="15" x14ac:dyDescent="0.2">
+      <c r="A15" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="B15" s="7" t="s">
+        <v>458</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2" ht="15" x14ac:dyDescent="0.2">
+      <c r="A16" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="B16" s="4" t="s">
+        <v>462</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2" ht="15" x14ac:dyDescent="0.2">
+      <c r="A17" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="B17" s="7" t="s">
+        <v>463</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" ht="15" x14ac:dyDescent="0.2">
+      <c r="A18" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="B18" s="7" t="s">
+        <v>464</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" ht="15" x14ac:dyDescent="0.2">
+      <c r="A19" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="B19" s="4" t="s">
+        <v>465</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2" ht="15" x14ac:dyDescent="0.2">
+      <c r="A20" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="B20" s="4" t="s">
+        <v>466</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" ht="15" x14ac:dyDescent="0.2">
+      <c r="A21" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="B21" s="4" t="s">
+        <v>467</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" ht="15" x14ac:dyDescent="0.2">
+      <c r="A22" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="B22" s="4" t="s">
+        <v>468</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" ht="15" x14ac:dyDescent="0.2">
+      <c r="A23" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="B23" s="4" t="s">
+        <v>469</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2" ht="15" x14ac:dyDescent="0.2">
+      <c r="A24" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="B24" s="4" t="s">
+        <v>470</v>
+      </c>
+    </row>
+    <row r="25" spans="1:2" ht="15" x14ac:dyDescent="0.2">
+      <c r="A25" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="B25" s="4" t="s">
+        <v>471</v>
+      </c>
+    </row>
+    <row r="26" spans="1:2" ht="15" x14ac:dyDescent="0.2">
+      <c r="A26" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="B26" s="4" t="s">
+        <v>472</v>
+      </c>
+    </row>
+    <row r="27" spans="1:2" ht="15" x14ac:dyDescent="0.2">
+      <c r="A27" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="B27" s="4" t="s">
+        <v>473</v>
+      </c>
+    </row>
+    <row r="28" spans="1:2" ht="15" x14ac:dyDescent="0.2">
+      <c r="A28" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="B28" s="4" t="s">
+        <v>474</v>
+      </c>
+    </row>
+    <row r="29" spans="1:2" ht="15" x14ac:dyDescent="0.2">
+      <c r="A29" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="B29" s="4" t="s">
+        <v>475</v>
+      </c>
+    </row>
+    <row r="30" spans="1:2" ht="15" x14ac:dyDescent="0.2">
+      <c r="A30" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="B30" s="4" t="s">
+        <v>476</v>
+      </c>
+    </row>
+    <row r="31" spans="1:2" ht="15" x14ac:dyDescent="0.2">
+      <c r="A31" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="B31" s="4" t="s">
+        <v>477</v>
+      </c>
+    </row>
+    <row r="32" spans="1:2" ht="15" x14ac:dyDescent="0.2">
+      <c r="A32" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="B32" s="4" t="s">
+        <v>478</v>
+      </c>
+    </row>
+    <row r="33" spans="1:2" ht="15" x14ac:dyDescent="0.2">
+      <c r="A33" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="B33" s="4" t="s">
+        <v>479</v>
+      </c>
+    </row>
+    <row r="34" spans="1:2" ht="15" x14ac:dyDescent="0.2">
+      <c r="A34" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="B34" s="4" t="s">
+        <v>480</v>
+      </c>
+    </row>
+    <row r="35" spans="1:2" ht="15" x14ac:dyDescent="0.2">
+      <c r="A35" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="B35" s="4" t="s">
+        <v>481</v>
+      </c>
+    </row>
+    <row r="36" spans="1:2" ht="15" x14ac:dyDescent="0.2">
+      <c r="A36" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="B36" s="4" t="s">
+        <v>482</v>
+      </c>
+    </row>
+    <row r="37" spans="1:2" ht="15" x14ac:dyDescent="0.2">
+      <c r="A37" s="3" t="s">
+        <v>536</v>
+      </c>
+      <c r="B37" s="4" t="s">
+        <v>538</v>
+      </c>
+    </row>
+    <row r="38" spans="1:2" ht="15" x14ac:dyDescent="0.2">
+      <c r="A38" s="3" t="s">
+        <v>537</v>
+      </c>
+      <c r="B38" s="4" t="s">
+        <v>539</v>
+      </c>
+    </row>
+    <row r="39" spans="1:2" ht="15" x14ac:dyDescent="0.2">
+      <c r="A39" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="B39" s="4" t="s">
+        <v>483</v>
+      </c>
+    </row>
+    <row r="40" spans="1:2" ht="15" x14ac:dyDescent="0.2">
+      <c r="A40" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="B40" s="4" t="s">
+        <v>484</v>
+      </c>
+    </row>
+    <row r="41" spans="1:2" ht="15" x14ac:dyDescent="0.2">
+      <c r="A41" s="3" t="s">
+        <v>541</v>
+      </c>
+      <c r="B41" s="4" t="s">
+        <v>545</v>
+      </c>
+    </row>
+    <row r="42" spans="1:2" ht="15" x14ac:dyDescent="0.2">
+      <c r="A42" s="3" t="s">
+        <v>542</v>
+      </c>
+      <c r="B42" s="4" t="s">
+        <v>485</v>
+      </c>
+    </row>
+    <row r="43" spans="1:2" ht="15" x14ac:dyDescent="0.2">
+      <c r="A43" s="3" t="s">
+        <v>540</v>
+      </c>
+      <c r="B43" s="4" t="s">
+        <v>544</v>
+      </c>
+    </row>
+    <row r="44" spans="1:2" ht="15" x14ac:dyDescent="0.2">
+      <c r="A44" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="B44" s="4" t="s">
+        <v>486</v>
+      </c>
+    </row>
+    <row r="45" spans="1:2" ht="15" x14ac:dyDescent="0.2">
+      <c r="A45" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="B45" s="4" t="s">
+        <v>487</v>
+      </c>
+    </row>
+    <row r="46" spans="1:2" ht="15" x14ac:dyDescent="0.2">
+      <c r="A46" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="B46" s="4" t="s">
+        <v>488</v>
+      </c>
+    </row>
+    <row r="47" spans="1:2" ht="15" x14ac:dyDescent="0.2">
+      <c r="A47" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="B47" s="4" t="s">
+        <v>489</v>
+      </c>
+    </row>
+    <row r="48" spans="1:2" ht="15" x14ac:dyDescent="0.2">
+      <c r="A48" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="B48" s="4" t="s">
+        <v>490</v>
+      </c>
+    </row>
+    <row r="49" spans="1:2" ht="15" x14ac:dyDescent="0.2">
+      <c r="A49" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="B49" s="4" t="s">
+        <v>491</v>
+      </c>
+    </row>
+    <row r="50" spans="1:2" ht="15" x14ac:dyDescent="0.2">
+      <c r="A50" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="B50" s="4" t="s">
+        <v>488</v>
+      </c>
+    </row>
+    <row r="51" spans="1:2" ht="15" x14ac:dyDescent="0.2">
+      <c r="A51" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="B51" s="4" t="s">
+        <v>489</v>
+      </c>
+    </row>
+    <row r="52" spans="1:2" ht="15" x14ac:dyDescent="0.2">
+      <c r="A52" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="B52" s="4" t="s">
+        <v>492</v>
+      </c>
+    </row>
+    <row r="53" spans="1:2" ht="15" x14ac:dyDescent="0.2">
+      <c r="A53" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="B53" s="4" t="s">
+        <v>493</v>
+      </c>
+    </row>
+    <row r="54" spans="1:2" ht="15" x14ac:dyDescent="0.2">
+      <c r="A54" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="B54" s="4" t="s">
+        <v>492</v>
+      </c>
+    </row>
+    <row r="55" spans="1:2" ht="15" x14ac:dyDescent="0.2">
+      <c r="A55" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="B55" s="4" t="s">
+        <v>493</v>
+      </c>
+    </row>
+    <row r="56" spans="1:2" ht="15" x14ac:dyDescent="0.2">
+      <c r="A56" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="B56" s="4" t="s">
+        <v>494</v>
+      </c>
+    </row>
+    <row r="57" spans="1:2" ht="15" x14ac:dyDescent="0.2">
+      <c r="A57" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="B57" s="4" t="s">
+        <v>495</v>
+      </c>
+    </row>
+    <row r="58" spans="1:2" ht="15" x14ac:dyDescent="0.2">
+      <c r="A58" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="B58" s="4" t="s">
+        <v>496</v>
+      </c>
+    </row>
+    <row r="59" spans="1:2" ht="15" x14ac:dyDescent="0.2">
+      <c r="A59" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="B59" s="4" t="s">
+        <v>497</v>
+      </c>
+    </row>
+    <row r="60" spans="1:2" ht="15" x14ac:dyDescent="0.2">
+      <c r="A60" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="B60" s="4" t="s">
+        <v>498</v>
+      </c>
+    </row>
+    <row r="61" spans="1:2" ht="15" x14ac:dyDescent="0.2">
+      <c r="A61" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="B61" s="4" t="s">
+        <v>499</v>
+      </c>
+    </row>
+    <row r="62" spans="1:2" ht="15" x14ac:dyDescent="0.2">
+      <c r="A62" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="B62" s="4" t="s">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="63" spans="1:2" ht="15" x14ac:dyDescent="0.2">
+      <c r="A63" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="B63" s="4" t="s">
+        <v>501</v>
+      </c>
+    </row>
+    <row r="64" spans="1:2" ht="15" x14ac:dyDescent="0.2">
+      <c r="A64" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="B64" s="4" t="s">
+        <v>502</v>
+      </c>
+    </row>
+    <row r="65" spans="1:2" ht="15" x14ac:dyDescent="0.2">
+      <c r="A65" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="B65" s="4" t="s">
+        <v>503</v>
+      </c>
+    </row>
+    <row r="66" spans="1:2" ht="15" x14ac:dyDescent="0.2">
+      <c r="A66" s="3" t="s">
+        <v>55</v>
+      </c>
+      <c r="B66" s="4" t="s">
+        <v>504</v>
+      </c>
+    </row>
+    <row r="67" spans="1:2" ht="15" x14ac:dyDescent="0.2">
+      <c r="A67" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="B67" s="4" t="s">
+        <v>505</v>
+      </c>
+    </row>
+    <row r="68" spans="1:2" ht="15" x14ac:dyDescent="0.2">
+      <c r="A68" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="B68" s="4" t="s">
+        <v>506</v>
+      </c>
+    </row>
+    <row r="69" spans="1:2" ht="15" x14ac:dyDescent="0.2">
+      <c r="A69" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="B69" s="4" t="s">
+        <v>507</v>
+      </c>
+    </row>
+    <row r="70" spans="1:2" ht="15" x14ac:dyDescent="0.2">
+      <c r="A70" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="B70" s="4" t="s">
+        <v>508</v>
+      </c>
+    </row>
+    <row r="71" spans="1:2" ht="15" x14ac:dyDescent="0.2">
+      <c r="A71" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="B71" s="4" t="s">
+        <v>509</v>
+      </c>
+    </row>
+    <row r="72" spans="1:2" ht="15" x14ac:dyDescent="0.2">
+      <c r="A72" s="3" t="s">
+        <v>61</v>
+      </c>
+      <c r="B72" s="4" t="s">
+        <v>510</v>
+      </c>
+    </row>
+    <row r="73" spans="1:2" ht="15" x14ac:dyDescent="0.2">
+      <c r="A73" s="3" t="s">
+        <v>62</v>
+      </c>
+      <c r="B73" s="4" t="s">
+        <v>511</v>
+      </c>
+    </row>
+    <row r="74" spans="1:2" ht="15" x14ac:dyDescent="0.2">
+      <c r="A74" s="3" t="s">
+        <v>71</v>
+      </c>
+      <c r="B74" s="4" t="s">
+        <v>512</v>
+      </c>
+    </row>
+    <row r="75" spans="1:2" ht="15" x14ac:dyDescent="0.2">
+      <c r="A75" s="3" t="s">
+        <v>72</v>
+      </c>
+      <c r="B75" s="4" t="s">
+        <v>513</v>
+      </c>
+    </row>
+    <row r="76" spans="1:2" ht="15" x14ac:dyDescent="0.2">
+      <c r="A76" s="3" t="s">
+        <v>69</v>
+      </c>
+      <c r="B76" s="4" t="s">
+        <v>514</v>
+      </c>
+    </row>
+    <row r="77" spans="1:2" ht="15" x14ac:dyDescent="0.2">
+      <c r="A77" s="3" t="s">
+        <v>70</v>
+      </c>
+      <c r="B77" s="4" t="s">
+        <v>515</v>
+      </c>
+    </row>
+    <row r="78" spans="1:2" ht="15" x14ac:dyDescent="0.2">
+      <c r="A78" s="3" t="s">
+        <v>63</v>
+      </c>
+      <c r="B78" s="4" t="s">
+        <v>516</v>
+      </c>
+    </row>
+    <row r="79" spans="1:2" ht="15" x14ac:dyDescent="0.2">
+      <c r="A79" s="3" t="s">
+        <v>64</v>
+      </c>
+      <c r="B79" s="4" t="s">
+        <v>517</v>
+      </c>
+    </row>
+    <row r="80" spans="1:2" ht="15" x14ac:dyDescent="0.2">
+      <c r="A80" s="3" t="s">
+        <v>67</v>
+      </c>
+      <c r="B80" s="4" t="s">
+        <v>518</v>
+      </c>
+    </row>
+    <row r="81" spans="1:4" ht="15" x14ac:dyDescent="0.2">
+      <c r="A81" s="3" t="s">
+        <v>68</v>
+      </c>
+      <c r="B81" s="4" t="s">
+        <v>519</v>
+      </c>
+    </row>
+    <row r="82" spans="1:4" ht="15" x14ac:dyDescent="0.2">
+      <c r="A82" s="3" t="s">
+        <v>65</v>
+      </c>
+      <c r="B82" s="4" t="s">
+        <v>520</v>
+      </c>
+    </row>
+    <row r="83" spans="1:4" ht="15" x14ac:dyDescent="0.2">
+      <c r="A83" s="3" t="s">
+        <v>66</v>
+      </c>
+      <c r="B83" s="4" t="s">
+        <v>521</v>
+      </c>
+    </row>
+    <row r="84" spans="1:4" ht="15" x14ac:dyDescent="0.2">
+      <c r="A84" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="B84" s="4" t="s">
+        <v>522</v>
+      </c>
+    </row>
+    <row r="85" spans="1:4" ht="15" x14ac:dyDescent="0.2">
+      <c r="A85" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="B85" s="4" t="s">
+        <v>523</v>
+      </c>
+    </row>
+    <row r="86" spans="1:4" ht="15" x14ac:dyDescent="0.2">
+      <c r="A86" s="3" t="s">
+        <v>73</v>
+      </c>
+      <c r="B86" s="4" t="s">
+        <v>524</v>
+      </c>
+    </row>
+    <row r="87" spans="1:4" ht="15" x14ac:dyDescent="0.2">
+      <c r="A87" s="3" t="s">
+        <v>74</v>
+      </c>
+      <c r="B87" s="4" t="s">
+        <v>525</v>
+      </c>
+    </row>
+    <row r="88" spans="1:4" ht="15" x14ac:dyDescent="0.2">
+      <c r="A88" s="3" t="s">
+        <v>75</v>
+      </c>
+      <c r="B88" s="4" t="s">
+        <v>526</v>
+      </c>
+    </row>
+    <row r="89" spans="1:4" ht="15" x14ac:dyDescent="0.2">
+      <c r="A89" s="3" t="s">
+        <v>76</v>
+      </c>
+      <c r="B89" s="4" t="s">
+        <v>527</v>
+      </c>
+    </row>
+    <row r="90" spans="1:4" ht="15" x14ac:dyDescent="0.2">
+      <c r="A90" s="3" t="s">
+        <v>77</v>
+      </c>
+      <c r="B90" s="4" t="s">
+        <v>528</v>
+      </c>
+    </row>
+    <row r="91" spans="1:4" ht="15" x14ac:dyDescent="0.2">
+      <c r="A91" s="3" t="s">
+        <v>78</v>
+      </c>
+      <c r="B91" s="4" t="s">
+        <v>529</v>
+      </c>
+    </row>
+    <row r="92" spans="1:4" ht="15" x14ac:dyDescent="0.2">
+      <c r="A92" s="3" t="s">
+        <v>79</v>
+      </c>
+      <c r="B92" s="4" t="s">
+        <v>530</v>
+      </c>
+    </row>
+    <row r="93" spans="1:4" ht="15" x14ac:dyDescent="0.2">
+      <c r="A93" s="3" t="s">
+        <v>80</v>
+      </c>
+      <c r="B93" s="4" t="s">
+        <v>531</v>
+      </c>
+    </row>
+    <row r="94" spans="1:4" ht="15" x14ac:dyDescent="0.2">
+      <c r="A94" s="3" t="s">
+        <v>81</v>
+      </c>
+      <c r="B94" s="4" t="s">
+        <v>532</v>
+      </c>
+    </row>
+    <row r="95" spans="1:4" ht="15" x14ac:dyDescent="0.2">
+      <c r="A95" s="3" t="s">
+        <v>82</v>
+      </c>
+      <c r="B95" s="4" t="s">
+        <v>533</v>
+      </c>
+    </row>
+    <row r="96" spans="1:4" ht="15" x14ac:dyDescent="0.2">
+      <c r="A96" s="8" t="s">
+        <v>83</v>
+      </c>
+      <c r="B96" s="5" t="s">
+        <v>534</v>
+      </c>
+      <c r="C96" s="1"/>
+      <c r="D96" s="1"/>
+    </row>
+    <row r="97" spans="1:4" ht="15" x14ac:dyDescent="0.2">
+      <c r="A97" s="9" t="s">
+        <v>84</v>
+      </c>
+      <c r="B97" s="5" t="s">
+        <v>535</v>
+      </c>
+      <c r="C97" s="1"/>
+      <c r="D97" s="1"/>
+    </row>
+    <row r="104" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A104" s="3"/>
+      <c r="B104" s="4"/>
+    </row>
+    <row r="105" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A105" s="3"/>
+      <c r="B105" s="4"/>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:B1"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>